<commit_message>
3.3 Tracking Error Minimization
</commit_message>
<xml_diff>
--- a/results/monthly_returns.xlsx
+++ b/results/monthly_returns.xlsx
@@ -20,13 +20,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,13 +48,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -421,453 +435,453 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>VW</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>MVP</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" s="2" t="n">
         <v>41670</v>
       </c>
       <c r="B2" t="n">
         <v>-0.03577051251348723</v>
       </c>
       <c r="C2" t="n">
-        <v>2.730222653150524e-06</v>
+        <v>2.730222653296241e-06</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" s="2" t="n">
         <v>41698</v>
       </c>
       <c r="B3" t="n">
         <v>0.05457272646088732</v>
       </c>
       <c r="C3" t="n">
-        <v>0.04891788266058264</v>
+        <v>0.04891788266058272</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" s="2" t="n">
         <v>41729</v>
       </c>
       <c r="B4" t="n">
         <v>0.007762261335563271</v>
       </c>
       <c r="C4" t="n">
-        <v>0.00297622123096899</v>
+        <v>0.002976221230969092</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" s="2" t="n">
         <v>41759</v>
       </c>
       <c r="B5" t="n">
         <v>0.01583202208543277</v>
       </c>
       <c r="C5" t="n">
-        <v>0.01963062223914377</v>
+        <v>0.01963062223914375</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" s="2" t="n">
         <v>41789</v>
       </c>
       <c r="B6" t="n">
         <v>0.01643020929599076</v>
       </c>
       <c r="C6" t="n">
-        <v>0.007681447610686071</v>
+        <v>0.007681447610686079</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" s="2" t="n">
         <v>41820</v>
       </c>
       <c r="B7" t="n">
         <v>0.01148059602195001</v>
       </c>
       <c r="C7" t="n">
-        <v>0.005367108850342425</v>
+        <v>0.005367108850342378</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" s="2" t="n">
         <v>41851</v>
       </c>
       <c r="B8" t="n">
         <v>-0.023164508181366</v>
       </c>
       <c r="C8" t="n">
-        <v>-0.04029218519291371</v>
+        <v>-0.04029218519291357</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" s="2" t="n">
         <v>41880</v>
       </c>
       <c r="B9" t="n">
         <v>0.02457691833184666</v>
       </c>
       <c r="C9" t="n">
-        <v>0.02976601488670137</v>
+        <v>0.02976601488670122</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" s="2" t="n">
         <v>41912</v>
       </c>
       <c r="B10" t="n">
         <v>-0.02330935776278098</v>
       </c>
       <c r="C10" t="n">
-        <v>-0.0390522615359757</v>
+        <v>-0.03905226153597566</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" s="2" t="n">
         <v>41943</v>
       </c>
       <c r="B11" t="n">
         <v>0.004941866289649032</v>
       </c>
       <c r="C11" t="n">
-        <v>0.04655124954081648</v>
+        <v>0.04655124954081642</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" s="2" t="n">
         <v>41971</v>
       </c>
       <c r="B12" t="n">
         <v>0.02684646801091424</v>
       </c>
       <c r="C12" t="n">
-        <v>0.03060666196916704</v>
+        <v>0.03060666196916687</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" s="2" t="n">
         <v>42004</v>
       </c>
       <c r="B13" t="n">
         <v>-0.01793837814404243</v>
       </c>
       <c r="C13" t="n">
-        <v>0.005229028925359563</v>
+        <v>0.005229028925359638</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" s="2" t="n">
         <v>42034</v>
       </c>
       <c r="B14" t="n">
         <v>-0.02282175733578628</v>
       </c>
       <c r="C14" t="n">
-        <v>0.003962826851777556</v>
+        <v>0.003962826851777302</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" s="2" t="n">
         <v>42062</v>
       </c>
       <c r="B15" t="n">
         <v>0.05685610170123574</v>
       </c>
       <c r="C15" t="n">
-        <v>0.00382872158217545</v>
+        <v>0.003828721582178348</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" s="2" t="n">
         <v>42094</v>
       </c>
       <c r="B16" t="n">
         <v>-0.01878225285036577</v>
       </c>
       <c r="C16" t="n">
-        <v>-0.01384128158688789</v>
+        <v>-0.01384128158689765</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
+      <c r="A17" s="2" t="n">
         <v>42124</v>
       </c>
       <c r="B17" t="n">
         <v>0.02217672013381462</v>
       </c>
       <c r="C17" t="n">
-        <v>0.002492671895549026</v>
+        <v>0.00249267189554782</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
+      <c r="A18" s="2" t="n">
         <v>42153</v>
       </c>
       <c r="B18" t="n">
         <v>0.002763819717271396</v>
       </c>
       <c r="C18" t="n">
-        <v>0.01117211679003133</v>
+        <v>0.01117211679002529</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
+      <c r="A19" s="2" t="n">
         <v>42185</v>
       </c>
       <c r="B19" t="n">
         <v>-0.02380750565336756</v>
       </c>
       <c r="C19" t="n">
-        <v>-0.02617371908367149</v>
+        <v>-0.02617371908367839</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
+      <c r="A20" s="2" t="n">
         <v>42216</v>
       </c>
       <c r="B20" t="n">
         <v>0.01953878974553074</v>
       </c>
       <c r="C20" t="n">
-        <v>0.04865401254992193</v>
+        <v>0.04865401254988987</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
+      <c r="A21" s="2" t="n">
         <v>42247</v>
       </c>
       <c r="B21" t="n">
         <v>-0.06371876922900283</v>
       </c>
       <c r="C21" t="n">
-        <v>-0.03001587259348153</v>
+        <v>-0.03001587259349209</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
+      <c r="A22" s="2" t="n">
         <v>42277</v>
       </c>
       <c r="B22" t="n">
         <v>-0.03029360394779007</v>
       </c>
       <c r="C22" t="n">
-        <v>-0.0127955190958921</v>
+        <v>-0.01279551909589483</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
+      <c r="A23" s="2" t="n">
         <v>42307</v>
       </c>
       <c r="B23" t="n">
         <v>0.07484781831623569</v>
       </c>
       <c r="C23" t="n">
-        <v>0.02227678680398361</v>
+        <v>0.02227678680400481</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
+      <c r="A24" s="2" t="n">
         <v>42338</v>
       </c>
       <c r="B24" t="n">
         <v>-0.005311215995536839</v>
       </c>
       <c r="C24" t="n">
-        <v>-0.006476912681995494</v>
+        <v>-0.006476912681978852</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
+      <c r="A25" s="2" t="n">
         <v>42369</v>
       </c>
       <c r="B25" t="n">
         <v>-0.02288379535149846</v>
       </c>
       <c r="C25" t="n">
-        <v>0.02650813033797372</v>
+        <v>0.02650813033797008</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
+      <c r="A26" s="2" t="n">
         <v>42398</v>
       </c>
       <c r="B26" t="n">
         <v>-0.05258465528398181</v>
       </c>
       <c r="C26" t="n">
-        <v>0.007202263417544447</v>
+        <v>0.007202263417535389</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
+      <c r="A27" s="2" t="n">
         <v>42429</v>
       </c>
       <c r="B27" t="n">
         <v>-0.008168481738206232</v>
       </c>
       <c r="C27" t="n">
-        <v>-0.004129525619341459</v>
+        <v>-0.004129525619331957</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
+      <c r="A28" s="2" t="n">
         <v>42460</v>
       </c>
       <c r="B28" t="n">
         <v>0.07050360052854185</v>
       </c>
       <c r="C28" t="n">
-        <v>0.04860880597788868</v>
+        <v>0.04860880597789544</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
+      <c r="A29" s="2" t="n">
         <v>42489</v>
       </c>
       <c r="B29" t="n">
         <v>0.01346581614572162</v>
       </c>
       <c r="C29" t="n">
-        <v>0.01856700237040105</v>
+        <v>0.01856700237040006</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="n">
+      <c r="A30" s="2" t="n">
         <v>42521</v>
       </c>
       <c r="B30" t="n">
         <v>0.00659258352088357</v>
       </c>
       <c r="C30" t="n">
-        <v>0.01027099558763282</v>
+        <v>0.01027099558763584</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="n">
+      <c r="A31" s="2" t="n">
         <v>42551</v>
       </c>
       <c r="B31" t="n">
         <v>-0.01362076122737209</v>
       </c>
       <c r="C31" t="n">
-        <v>0.0570116054128005</v>
+        <v>0.05701160541280054</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="n">
+      <c r="A32" s="2" t="n">
         <v>42580</v>
       </c>
       <c r="B32" t="n">
         <v>0.03674407370358323</v>
       </c>
       <c r="C32" t="n">
-        <v>0.02028425692059983</v>
+        <v>0.02028425692060203</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="n">
+      <c r="A33" s="2" t="n">
         <v>42613</v>
       </c>
       <c r="B33" t="n">
         <v>0.002077100500778767</v>
       </c>
       <c r="C33" t="n">
-        <v>-0.04585631771578419</v>
+        <v>-0.04585631771577894</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="n">
+      <c r="A34" s="2" t="n">
         <v>42643</v>
       </c>
       <c r="B34" t="n">
         <v>0.002306627011404471</v>
       </c>
       <c r="C34" t="n">
-        <v>-0.01514616317556679</v>
+        <v>-0.01514616317556969</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="n">
+      <c r="A35" s="2" t="n">
         <v>42674</v>
       </c>
       <c r="B35" t="n">
         <v>-0.02102440381119557</v>
       </c>
       <c r="C35" t="n">
-        <v>-0.03581039563152387</v>
+        <v>-0.03581039563151144</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="n">
+      <c r="A36" s="2" t="n">
         <v>42704</v>
       </c>
       <c r="B36" t="n">
         <v>0.01819181100066963</v>
       </c>
       <c r="C36" t="n">
-        <v>-0.02037946179393673</v>
+        <v>-0.0203794617939423</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="n">
+      <c r="A37" s="2" t="n">
         <v>42734</v>
       </c>
       <c r="B37" t="n">
         <v>0.03324819018946118</v>
       </c>
       <c r="C37" t="n">
-        <v>0.02901604237318179</v>
+        <v>0.02901604237318184</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="n">
+      <c r="A38" s="2" t="n">
         <v>42766</v>
       </c>
       <c r="B38" t="n">
         <v>0.01579079678590857</v>
       </c>
       <c r="C38" t="n">
-        <v>0.008000296440244394</v>
+        <v>0.008000296440244407</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n">
+      <c r="A39" s="2" t="n">
         <v>42794</v>
       </c>
       <c r="B39" t="n">
         <v>0.02844322118409615</v>
       </c>
       <c r="C39" t="n">
-        <v>0.02103760038850296</v>
+        <v>0.02103760038850297</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="n">
+      <c r="A40" s="2" t="n">
         <v>42825</v>
       </c>
       <c r="B40" t="n">
         <v>0.01407803634341376</v>
       </c>
       <c r="C40" t="n">
-        <v>0.003774695669464308</v>
+        <v>0.003774695669464323</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="n">
+      <c r="A41" s="2" t="n">
         <v>42853</v>
       </c>
       <c r="B41" t="n">
@@ -878,293 +892,293 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="n">
+      <c r="A42" s="2" t="n">
         <v>42886</v>
       </c>
       <c r="B42" t="n">
         <v>0.02654951259123661</v>
       </c>
       <c r="C42" t="n">
-        <v>0.03242084510237632</v>
+        <v>0.03242084510237631</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="n">
+      <c r="A43" s="2" t="n">
         <v>42916</v>
       </c>
       <c r="B43" t="n">
         <v>0.002373678903860118</v>
       </c>
       <c r="C43" t="n">
-        <v>-0.01179985612409165</v>
+        <v>-0.01179985612409164</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="n">
+      <c r="A44" s="2" t="n">
         <v>42947</v>
       </c>
       <c r="B44" t="n">
         <v>0.02246463779799775</v>
       </c>
       <c r="C44" t="n">
-        <v>0.02283386439866797</v>
+        <v>0.02283386439866803</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="n">
+      <c r="A45" s="2" t="n">
         <v>42978</v>
       </c>
       <c r="B45" t="n">
         <v>0.00244198517741814</v>
       </c>
       <c r="C45" t="n">
-        <v>-0.04791840198244822</v>
+        <v>-0.04791840198244816</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="n">
+      <c r="A46" s="2" t="n">
         <v>43007</v>
       </c>
       <c r="B46" t="n">
         <v>0.02808540905124245</v>
       </c>
       <c r="C46" t="n">
-        <v>0.008226210958247446</v>
+        <v>0.008226210958247351</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="n">
+      <c r="A47" s="2" t="n">
         <v>43039</v>
       </c>
       <c r="B47" t="n">
         <v>0.01894898151901998</v>
       </c>
       <c r="C47" t="n">
-        <v>0.01965537009971226</v>
+        <v>0.01965537009971235</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="n">
+      <c r="A48" s="2" t="n">
         <v>43069</v>
       </c>
       <c r="B48" t="n">
         <v>0.02194443635302347</v>
       </c>
       <c r="C48" t="n">
-        <v>0.03785084198989323</v>
+        <v>0.03785084198989316</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1" t="n">
+      <c r="A49" s="2" t="n">
         <v>43098</v>
       </c>
       <c r="B49" t="n">
         <v>0.01303863736857334</v>
       </c>
       <c r="C49" t="n">
-        <v>0.02080060156683984</v>
+        <v>0.02080060156683981</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1" t="n">
+      <c r="A50" s="2" t="n">
         <v>43131</v>
       </c>
       <c r="B50" t="n">
         <v>0.04951854951058408</v>
       </c>
       <c r="C50" t="n">
-        <v>-0.02108269564772578</v>
+        <v>-0.02108269564772554</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="n">
+      <c r="A51" s="2" t="n">
         <v>43159</v>
       </c>
       <c r="B51" t="n">
         <v>-0.04705500135027535</v>
       </c>
       <c r="C51" t="n">
-        <v>-0.07538499118428529</v>
+        <v>-0.07538499118428517</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1" t="n">
+      <c r="A52" s="2" t="n">
         <v>43189</v>
       </c>
       <c r="B52" t="n">
         <v>-0.01795301847933335</v>
       </c>
       <c r="C52" t="n">
-        <v>-0.006770242963501949</v>
+        <v>-0.006770242963501999</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="1" t="n">
+      <c r="A53" s="2" t="n">
         <v>43220</v>
       </c>
       <c r="B53" t="n">
         <v>0.01261748230660959</v>
       </c>
       <c r="C53" t="n">
-        <v>0.01037408419454142</v>
+        <v>0.0103740841945414</v>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="1" t="n">
+      <c r="A54" s="2" t="n">
         <v>43251</v>
       </c>
       <c r="B54" t="n">
         <v>0.001351174902387803</v>
       </c>
       <c r="C54" t="n">
-        <v>0.0008495935373884849</v>
+        <v>0.0008495935373884897</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="n">
+      <c r="A55" s="2" t="n">
         <v>43280</v>
       </c>
       <c r="B55" t="n">
         <v>0.0002616030988843816</v>
       </c>
       <c r="C55" t="n">
-        <v>0.01688277897535887</v>
+        <v>0.01688277897535898</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="1" t="n">
+      <c r="A56" s="2" t="n">
         <v>43312</v>
       </c>
       <c r="B56" t="n">
         <v>0.03849477634390881</v>
       </c>
       <c r="C56" t="n">
-        <v>0.007820125985214475</v>
+        <v>0.007820125985214546</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="1" t="n">
+      <c r="A57" s="2" t="n">
         <v>43343</v>
       </c>
       <c r="B57" t="n">
         <v>0.008992745924063218</v>
       </c>
       <c r="C57" t="n">
-        <v>0.03077127343045231</v>
+        <v>0.03077127343045237</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="1" t="n">
+      <c r="A58" s="2" t="n">
         <v>43371</v>
       </c>
       <c r="B58" t="n">
         <v>0.0066165392530823</v>
       </c>
       <c r="C58" t="n">
-        <v>-0.006763939976214378</v>
+        <v>-0.006763939976214333</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="1" t="n">
+      <c r="A59" s="2" t="n">
         <v>43404</v>
       </c>
       <c r="B59" t="n">
         <v>-0.06453623148170358</v>
       </c>
       <c r="C59" t="n">
-        <v>-0.008528733589575333</v>
+        <v>-0.008528733589575378</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="1" t="n">
+      <c r="A60" s="2" t="n">
         <v>43434</v>
       </c>
       <c r="B60" t="n">
         <v>0.01111789623001095</v>
       </c>
       <c r="C60" t="n">
-        <v>-0.02543711892555279</v>
+        <v>-0.02543711892555225</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="1" t="n">
+      <c r="A61" s="2" t="n">
         <v>43465</v>
       </c>
       <c r="B61" t="n">
         <v>-0.07816398564554208</v>
       </c>
       <c r="C61" t="n">
-        <v>-0.06309782624436892</v>
+        <v>-0.06309782624436877</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="1" t="n">
+      <c r="A62" s="2" t="n">
         <v>43496</v>
       </c>
       <c r="B62" t="n">
         <v>0.07601880736345278</v>
       </c>
       <c r="C62" t="n">
-        <v>0.01825868070332343</v>
+        <v>0.01825868070332333</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="1" t="n">
+      <c r="A63" s="2" t="n">
         <v>43524</v>
       </c>
       <c r="B63" t="n">
         <v>0.03326236662472595</v>
       </c>
       <c r="C63" t="n">
-        <v>0.03715013667570118</v>
+        <v>0.03715013667570122</v>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="1" t="n">
+      <c r="A64" s="2" t="n">
         <v>43553</v>
       </c>
       <c r="B64" t="n">
         <v>0.01472293864230933</v>
       </c>
       <c r="C64" t="n">
-        <v>0.0379509655422837</v>
+        <v>0.03795096554228373</v>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="1" t="n">
+      <c r="A65" s="2" t="n">
         <v>43585</v>
       </c>
       <c r="B65" t="n">
         <v>0.03766175186714266</v>
       </c>
       <c r="C65" t="n">
-        <v>0.03182501970714718</v>
+        <v>0.03182501970714726</v>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="1" t="n">
+      <c r="A66" s="2" t="n">
         <v>43616</v>
       </c>
       <c r="B66" t="n">
         <v>-0.06023474533191252</v>
       </c>
       <c r="C66" t="n">
-        <v>-0.01913396723817571</v>
+        <v>-0.01913396723817573</v>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="1" t="n">
+      <c r="A67" s="2" t="n">
         <v>43644</v>
       </c>
       <c r="B67" t="n">
         <v>0.07033903461068169</v>
       </c>
       <c r="C67" t="n">
-        <v>0.03889138671042734</v>
+        <v>0.03889138671042749</v>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="1" t="n">
+      <c r="A68" s="2" t="n">
         <v>43677</v>
       </c>
       <c r="B68" t="n">
@@ -1175,227 +1189,227 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="1" t="n">
+      <c r="A69" s="2" t="n">
         <v>43707</v>
       </c>
       <c r="B69" t="n">
         <v>-0.01828779657461423</v>
       </c>
       <c r="C69" t="n">
-        <v>0.006146565526305313</v>
+        <v>0.00614656552630522</v>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="1" t="n">
+      <c r="A70" s="2" t="n">
         <v>43738</v>
       </c>
       <c r="B70" t="n">
         <v>0.02466315429160364</v>
       </c>
       <c r="C70" t="n">
-        <v>0.01044742051010839</v>
+        <v>0.01044742051010836</v>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="1" t="n">
+      <c r="A71" s="2" t="n">
         <v>43769</v>
       </c>
       <c r="B71" t="n">
         <v>0.02217750538357088</v>
       </c>
       <c r="C71" t="n">
-        <v>-0.005609037583084731</v>
+        <v>-0.005609037583084878</v>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="1" t="n">
+      <c r="A72" s="2" t="n">
         <v>43798</v>
       </c>
       <c r="B72" t="n">
         <v>0.02997799889267743</v>
       </c>
       <c r="C72" t="n">
-        <v>0.01917680945616537</v>
+        <v>0.01917680945616541</v>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="1" t="n">
+      <c r="A73" s="2" t="n">
         <v>43830</v>
       </c>
       <c r="B73" t="n">
         <v>0.03482421028928007</v>
       </c>
       <c r="C73" t="n">
-        <v>0.04255413156750001</v>
+        <v>0.04255413156749994</v>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="1" t="n">
+      <c r="A74" s="2" t="n">
         <v>43861</v>
       </c>
       <c r="B74" t="n">
         <v>-0.009580265949088524</v>
       </c>
       <c r="C74" t="n">
-        <v>0.0140929927969088</v>
+        <v>0.01409299279690879</v>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="1" t="n">
+      <c r="A75" s="2" t="n">
         <v>43889</v>
       </c>
       <c r="B75" t="n">
         <v>-0.08791498768503248</v>
       </c>
       <c r="C75" t="n">
-        <v>-0.08525920946399373</v>
+        <v>-0.08525920946399368</v>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="1" t="n">
+      <c r="A76" s="2" t="n">
         <v>43921</v>
       </c>
       <c r="B76" t="n">
         <v>-0.1306650921429244</v>
       </c>
       <c r="C76" t="n">
-        <v>-0.124749125896036</v>
+        <v>-0.1247491258960358</v>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="1" t="n">
+      <c r="A77" s="2" t="n">
         <v>43951</v>
       </c>
       <c r="B77" t="n">
         <v>0.1075112783889687</v>
       </c>
       <c r="C77" t="n">
-        <v>0.111048518126205</v>
+        <v>0.1110485181262049</v>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="1" t="n">
+      <c r="A78" s="2" t="n">
         <v>43980</v>
       </c>
       <c r="B78" t="n">
         <v>0.04142078875265022</v>
       </c>
       <c r="C78" t="n">
-        <v>0.02457496452175811</v>
+        <v>0.02457496452175814</v>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="1" t="n">
+      <c r="A79" s="2" t="n">
         <v>44012</v>
       </c>
       <c r="B79" t="n">
         <v>0.02854315181783309</v>
       </c>
       <c r="C79" t="n">
-        <v>-0.009407842664746665</v>
+        <v>-0.009407842664746651</v>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="1" t="n">
+      <c r="A80" s="2" t="n">
         <v>44043</v>
       </c>
       <c r="B80" t="n">
         <v>0.04883592322798035</v>
       </c>
       <c r="C80" t="n">
-        <v>0.07388733025686636</v>
+        <v>0.07388733025686642</v>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="1" t="n">
+      <c r="A81" s="2" t="n">
         <v>44074</v>
       </c>
       <c r="B81" t="n">
         <v>0.06540930795489953</v>
       </c>
       <c r="C81" t="n">
-        <v>0.0347299651889283</v>
+        <v>0.03472996518892831</v>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="1" t="n">
+      <c r="A82" s="2" t="n">
         <v>44104</v>
       </c>
       <c r="B82" t="n">
         <v>-0.03798082063905267</v>
       </c>
       <c r="C82" t="n">
-        <v>-0.01828587876157299</v>
+        <v>-0.01828587876157301</v>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="1" t="n">
+      <c r="A83" s="2" t="n">
         <v>44134</v>
       </c>
       <c r="B83" t="n">
         <v>-0.03589474696672947</v>
       </c>
       <c r="C83" t="n">
-        <v>-0.018528846854483</v>
+        <v>-0.01852884685448301</v>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="1" t="n">
+      <c r="A84" s="2" t="n">
         <v>44165</v>
       </c>
       <c r="B84" t="n">
         <v>0.1283940181539289</v>
       </c>
       <c r="C84" t="n">
-        <v>0.07337263320928987</v>
+        <v>0.07337263320928981</v>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="1" t="n">
+      <c r="A85" s="2" t="n">
         <v>44196</v>
       </c>
       <c r="B85" t="n">
         <v>0.03983956548531003</v>
       </c>
       <c r="C85" t="n">
-        <v>0.02761180067773927</v>
+        <v>0.02761180067773917</v>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="1" t="n">
+      <c r="A86" s="2" t="n">
         <v>44225</v>
       </c>
       <c r="B86" t="n">
         <v>-0.01212400733186289</v>
       </c>
       <c r="C86" t="n">
-        <v>-0.008475547946880116</v>
+        <v>-0.00847554794687993</v>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="1" t="n">
+      <c r="A87" s="2" t="n">
         <v>44253</v>
       </c>
       <c r="B87" t="n">
         <v>0.02733062300679211</v>
       </c>
       <c r="C87" t="n">
-        <v>-0.0002929385122203247</v>
+        <v>-0.0002929385122206005</v>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="1" t="n">
+      <c r="A88" s="2" t="n">
         <v>44286</v>
       </c>
       <c r="B88" t="n">
         <v>0.04536283607748608</v>
       </c>
       <c r="C88" t="n">
-        <v>0.07860679864833137</v>
+        <v>0.07860679864833139</v>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="1" t="n">
+      <c r="A89" s="2" t="n">
         <v>44316</v>
       </c>
       <c r="B89" t="n">
@@ -1406,62 +1420,62 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="1" t="n">
+      <c r="A90" s="2" t="n">
         <v>44347</v>
       </c>
       <c r="B90" t="n">
         <v>0.02015621412882964</v>
       </c>
       <c r="C90" t="n">
-        <v>0.02586177073086889</v>
+        <v>0.02586177073086892</v>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="1" t="n">
+      <c r="A91" s="2" t="n">
         <v>44377</v>
       </c>
       <c r="B91" t="n">
         <v>0.009085467039068967</v>
       </c>
       <c r="C91" t="n">
-        <v>-0.0204594521137154</v>
+        <v>-0.02045945211371527</v>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="1" t="n">
+      <c r="A92" s="2" t="n">
         <v>44407</v>
       </c>
       <c r="B92" t="n">
         <v>0.01882876021698834</v>
       </c>
       <c r="C92" t="n">
-        <v>0.02666338376474656</v>
+        <v>0.02666338376474659</v>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="1" t="n">
+      <c r="A93" s="2" t="n">
         <v>44439</v>
       </c>
       <c r="B93" t="n">
         <v>0.02292599245632672</v>
       </c>
       <c r="C93" t="n">
-        <v>0.002387439376513915</v>
+        <v>0.002387439376513896</v>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="1" t="n">
+      <c r="A94" s="2" t="n">
         <v>44469</v>
       </c>
       <c r="B94" t="n">
         <v>-0.04484438196599666</v>
       </c>
       <c r="C94" t="n">
-        <v>-0.06122936085079829</v>
+        <v>-0.06122936085079826</v>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="1" t="n">
+      <c r="A95" s="2" t="n">
         <v>44498</v>
       </c>
       <c r="B95" t="n">
@@ -1472,205 +1486,205 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="1" t="n">
+      <c r="A96" s="2" t="n">
         <v>44530</v>
       </c>
       <c r="B96" t="n">
         <v>-0.01485364644369896</v>
       </c>
       <c r="C96" t="n">
-        <v>-0.03396186432802805</v>
+        <v>-0.03396186432802809</v>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="1" t="n">
+      <c r="A97" s="2" t="n">
         <v>44561</v>
       </c>
       <c r="B97" t="n">
         <v>0.05275242494481132</v>
       </c>
       <c r="C97" t="n">
-        <v>0.07491379473672632</v>
+        <v>0.07491379473672655</v>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="1" t="n">
+      <c r="A98" s="2" t="n">
         <v>44592</v>
       </c>
       <c r="B98" t="n">
         <v>-0.04101565747775374</v>
       </c>
       <c r="C98" t="n">
-        <v>-0.01040777410931138</v>
+        <v>-0.01040777410931704</v>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="1" t="n">
+      <c r="A99" s="2" t="n">
         <v>44620</v>
       </c>
       <c r="B99" t="n">
         <v>-0.02440661653703706</v>
       </c>
       <c r="C99" t="n">
-        <v>-0.0186504067041889</v>
+        <v>-0.0186504067041853</v>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="1" t="n">
+      <c r="A100" s="2" t="n">
         <v>44651</v>
       </c>
       <c r="B100" t="n">
         <v>0.02739841992527333</v>
       </c>
       <c r="C100" t="n">
-        <v>0.04370183673260911</v>
+        <v>0.04370183673260929</v>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="1" t="n">
+      <c r="A101" s="2" t="n">
         <v>44680</v>
       </c>
       <c r="B101" t="n">
         <v>-0.07246087523648355</v>
       </c>
       <c r="C101" t="n">
-        <v>-0.02808252545283147</v>
+        <v>-0.02808252545282783</v>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="1" t="n">
+      <c r="A102" s="2" t="n">
         <v>44712</v>
       </c>
       <c r="B102" t="n">
         <v>0.005871650263511217</v>
       </c>
       <c r="C102" t="n">
-        <v>0.01023325812738706</v>
+        <v>0.0102332581273923</v>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="1" t="n">
+      <c r="A103" s="2" t="n">
         <v>44742</v>
       </c>
       <c r="B103" t="n">
         <v>-0.08596805176643892</v>
       </c>
       <c r="C103" t="n">
-        <v>-0.05379045931736158</v>
+        <v>-0.05379045931733725</v>
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="1" t="n">
+      <c r="A104" s="2" t="n">
         <v>44771</v>
       </c>
       <c r="B104" t="n">
         <v>0.07919681433848735</v>
       </c>
       <c r="C104" t="n">
-        <v>0.02639147983837267</v>
+        <v>0.02639147983836548</v>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="1" t="n">
+      <c r="A105" s="2" t="n">
         <v>44804</v>
       </c>
       <c r="B105" t="n">
         <v>-0.04332771130830771</v>
       </c>
       <c r="C105" t="n">
-        <v>-0.03353423439715109</v>
+        <v>-0.03353423439714249</v>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="1" t="n">
+      <c r="A106" s="2" t="n">
         <v>44834</v>
       </c>
       <c r="B106" t="n">
         <v>-0.09169976227284632</v>
       </c>
       <c r="C106" t="n">
-        <v>-0.08064395506674363</v>
+        <v>-0.08064395506676628</v>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="1" t="n">
+      <c r="A107" s="2" t="n">
         <v>44865</v>
       </c>
       <c r="B107" t="n">
         <v>0.08600326884212639</v>
       </c>
       <c r="C107" t="n">
-        <v>0.06432684165014646</v>
+        <v>0.06432684165012396</v>
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="1" t="n">
+      <c r="A108" s="2" t="n">
         <v>44895</v>
       </c>
       <c r="B108" t="n">
         <v>0.07019817439074505</v>
       </c>
       <c r="C108" t="n">
-        <v>0.05811044115169554</v>
+        <v>0.05811044115168718</v>
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="1" t="n">
+      <c r="A109" s="2" t="n">
         <v>44925</v>
       </c>
       <c r="B109" t="n">
         <v>-0.04196388752670809</v>
       </c>
       <c r="C109" t="n">
-        <v>-0.02738915085563594</v>
+        <v>-0.02738915085564868</v>
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="1" t="n">
+      <c r="A110" s="2" t="n">
         <v>44957</v>
       </c>
       <c r="B110" t="n">
         <v>0.06616089743523371</v>
       </c>
       <c r="C110" t="n">
-        <v>0.02469967352489349</v>
+        <v>0.02469967352489337</v>
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="1" t="n">
+      <c r="A111" s="2" t="n">
         <v>44985</v>
       </c>
       <c r="B111" t="n">
         <v>-0.02239431803222399</v>
       </c>
       <c r="C111" t="n">
-        <v>-0.00289158671728222</v>
+        <v>-0.002891586717282327</v>
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="1" t="n">
+      <c r="A112" s="2" t="n">
         <v>45016</v>
       </c>
       <c r="B112" t="n">
         <v>0.03122580989791321</v>
       </c>
       <c r="C112" t="n">
-        <v>0.01357216473408979</v>
+        <v>0.01357216473408997</v>
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="1" t="n">
+      <c r="A113" s="2" t="n">
         <v>45044</v>
       </c>
       <c r="B113" t="n">
         <v>0.02644255003476621</v>
       </c>
       <c r="C113" t="n">
-        <v>0.02665806870843073</v>
+        <v>0.0266580687084309</v>
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="1" t="n">
+      <c r="A114" s="2" t="n">
         <v>45077</v>
       </c>
       <c r="B114" t="n">
@@ -1681,238 +1695,238 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="1" t="n">
+      <c r="A115" s="2" t="n">
         <v>45107</v>
       </c>
       <c r="B115" t="n">
         <v>0.06093188600225954</v>
       </c>
       <c r="C115" t="n">
-        <v>0.01356101307124157</v>
+        <v>0.01356101307124181</v>
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="1" t="n">
+      <c r="A116" s="2" t="n">
         <v>45138</v>
       </c>
       <c r="B116" t="n">
         <v>0.0290835962367811</v>
       </c>
       <c r="C116" t="n">
-        <v>0.007779183779411554</v>
+        <v>0.007779183779411563</v>
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="1" t="n">
+      <c r="A117" s="2" t="n">
         <v>45169</v>
       </c>
       <c r="B117" t="n">
         <v>-0.02253641802697804</v>
       </c>
       <c r="C117" t="n">
-        <v>-0.01816153083576303</v>
+        <v>-0.01816153083576296</v>
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="1" t="n">
+      <c r="A118" s="2" t="n">
         <v>45198</v>
       </c>
       <c r="B118" t="n">
         <v>-0.04645542708300802</v>
       </c>
       <c r="C118" t="n">
-        <v>-0.04695878780422914</v>
+        <v>-0.0469587878042293</v>
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="1" t="n">
+      <c r="A119" s="2" t="n">
         <v>45230</v>
       </c>
       <c r="B119" t="n">
         <v>-0.02171054624420314</v>
       </c>
       <c r="C119" t="n">
-        <v>-0.007236148857404152</v>
+        <v>-0.007236148857404119</v>
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="1" t="n">
+      <c r="A120" s="2" t="n">
         <v>45260</v>
       </c>
       <c r="B120" t="n">
         <v>0.09051414707262974</v>
       </c>
       <c r="C120" t="n">
-        <v>0.02714817936583027</v>
+        <v>0.02714817936583044</v>
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="1" t="n">
+      <c r="A121" s="2" t="n">
         <v>45289</v>
       </c>
       <c r="B121" t="n">
         <v>0.04513240680873794</v>
       </c>
       <c r="C121" t="n">
-        <v>0.01303706415322584</v>
+        <v>0.01303706415322593</v>
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="1" t="n">
+      <c r="A122" s="2" t="n">
         <v>45322</v>
       </c>
       <c r="B122" t="n">
         <v>0.01245418746238778</v>
       </c>
       <c r="C122" t="n">
-        <v>-0.009093756460089478</v>
+        <v>-0.009093756460092309</v>
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="1" t="n">
+      <c r="A123" s="2" t="n">
         <v>45351</v>
       </c>
       <c r="B123" t="n">
         <v>0.03901825082531514</v>
       </c>
       <c r="C123" t="n">
-        <v>0.0359489109885649</v>
+        <v>0.03594891098855772</v>
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="1" t="n">
+      <c r="A124" s="2" t="n">
         <v>45380</v>
       </c>
       <c r="B124" t="n">
         <v>0.03637442820614256</v>
       </c>
       <c r="C124" t="n">
-        <v>0.02523437034638502</v>
+        <v>0.02523437034638649</v>
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="1" t="n">
+      <c r="A125" s="2" t="n">
         <v>45412</v>
       </c>
       <c r="B125" t="n">
         <v>-0.03609511822437324</v>
       </c>
       <c r="C125" t="n">
-        <v>0.019047899332591</v>
+        <v>0.01904789933259306</v>
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="1" t="n">
+      <c r="A126" s="2" t="n">
         <v>45443</v>
       </c>
       <c r="B126" t="n">
         <v>0.05159895294222033</v>
       </c>
       <c r="C126" t="n">
-        <v>0.02202757570791411</v>
+        <v>0.02202757570791832</v>
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="1" t="n">
+      <c r="A127" s="2" t="n">
         <v>45471</v>
       </c>
       <c r="B127" t="n">
         <v>0.01673400189527829</v>
       </c>
       <c r="C127" t="n">
-        <v>-0.01700788360700735</v>
+        <v>-0.01700788360701016</v>
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="1" t="n">
+      <c r="A128" s="2" t="n">
         <v>45504</v>
       </c>
       <c r="B128" t="n">
         <v>0.01638886236175519</v>
       </c>
       <c r="C128" t="n">
-        <v>0.02504571085099025</v>
+        <v>0.02504571085099221</v>
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="1" t="n">
+      <c r="A129" s="2" t="n">
         <v>45534</v>
       </c>
       <c r="B129" t="n">
         <v>0.02662711852757172</v>
       </c>
       <c r="C129" t="n">
-        <v>0.03280900611414459</v>
+        <v>0.03280900611413946</v>
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="1" t="n">
+      <c r="A130" s="2" t="n">
         <v>45565</v>
       </c>
       <c r="B130" t="n">
         <v>0.01491367792089069</v>
       </c>
       <c r="C130" t="n">
-        <v>-0.005177790269040688</v>
+        <v>-0.005177790269040606</v>
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="1" t="n">
+      <c r="A131" s="2" t="n">
         <v>45596</v>
       </c>
       <c r="B131" t="n">
         <v>-0.02230215658726872</v>
       </c>
       <c r="C131" t="n">
-        <v>-0.0444944105699073</v>
+        <v>-0.0444944105699025</v>
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="1" t="n">
+      <c r="A132" s="2" t="n">
         <v>45625</v>
       </c>
       <c r="B132" t="n">
         <v>0.04154212052715963</v>
       </c>
       <c r="C132" t="n">
-        <v>-0.006102921933921876</v>
+        <v>-0.006102921933923455</v>
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="1" t="n">
+      <c r="A133" s="2" t="n">
         <v>45657</v>
       </c>
       <c r="B133" t="n">
         <v>-0.03216767101109499</v>
       </c>
       <c r="C133" t="n">
-        <v>-0.02658561534534414</v>
+        <v>-0.02658561534534758</v>
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="1" t="n">
+      <c r="A134" s="2" t="n">
         <v>45688</v>
       </c>
       <c r="B134" t="n">
         <v>0.03074400383563204</v>
       </c>
       <c r="C134" t="n">
-        <v>-0.006027115472455921</v>
+        <v>-0.006027115472455938</v>
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="1" t="n">
+      <c r="A135" s="2" t="n">
         <v>45716</v>
       </c>
       <c r="B135" t="n">
         <v>0.005356171982461908</v>
       </c>
       <c r="C135" t="n">
-        <v>0.005306823159101683</v>
+        <v>0.00530682315910169</v>
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="1" t="n">
+      <c r="A136" s="2" t="n">
         <v>45747</v>
       </c>
       <c r="B136" t="n">
@@ -1923,102 +1937,102 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="1" t="n">
+      <c r="A137" s="2" t="n">
         <v>45777</v>
       </c>
       <c r="B137" t="n">
         <v>-0.0003712512432697251</v>
       </c>
       <c r="C137" t="n">
-        <v>0.04393901351277293</v>
+        <v>0.04393901351277295</v>
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="1" t="n">
+      <c r="A138" s="2" t="n">
         <v>45807</v>
       </c>
       <c r="B138" t="n">
         <v>0.05049871444190139</v>
       </c>
       <c r="C138" t="n">
-        <v>-0.01871251790217808</v>
+        <v>-0.01871251790217802</v>
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="1" t="n">
+      <c r="A139" s="2" t="n">
         <v>45838</v>
       </c>
       <c r="B139" t="n">
         <v>0.043684099601013</v>
       </c>
       <c r="C139" t="n">
-        <v>-0.007032588549490621</v>
+        <v>-0.00703258854949062</v>
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="1" t="n">
+      <c r="A140" s="2" t="n">
         <v>45869</v>
       </c>
       <c r="B140" t="n">
         <v>0.01704349688554993</v>
       </c>
       <c r="C140" t="n">
-        <v>-0.003793539940815096</v>
+        <v>-0.003793539940815127</v>
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="1" t="n">
+      <c r="A141" s="2" t="n">
         <v>45898</v>
       </c>
       <c r="B141" t="n">
         <v>0.02376419689285764</v>
       </c>
       <c r="C141" t="n">
-        <v>0.009855526705872263</v>
+        <v>0.009855526705872236</v>
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="1" t="n">
+      <c r="A142" s="2" t="n">
         <v>45930</v>
       </c>
       <c r="B142" t="n">
         <v>0.02752594267972975</v>
       </c>
       <c r="C142" t="n">
-        <v>0.004432415254182327</v>
+        <v>0.004432415254182237</v>
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="1" t="n">
+      <c r="A143" s="2" t="n">
         <v>45961</v>
       </c>
       <c r="B143" t="n">
         <v>0.02345311271306457</v>
       </c>
       <c r="C143" t="n">
-        <v>-0.01505123076461782</v>
+        <v>-0.0150512307646178</v>
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="1" t="n">
+      <c r="A144" s="2" t="n">
         <v>45989</v>
       </c>
       <c r="B144" t="n">
         <v>0.007211569097595304</v>
       </c>
       <c r="C144" t="n">
-        <v>0.05424916396365365</v>
+        <v>0.05424916396365363</v>
       </c>
     </row>
     <row r="145">
-      <c r="A145" s="1" t="n">
+      <c r="A145" s="2" t="n">
         <v>46022</v>
       </c>
       <c r="B145" t="n">
         <v>0.0145794998106231</v>
       </c>
       <c r="C145" t="n">
-        <v>0.00386860095134728</v>
+        <v>0.003868600951347357</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
More or less code is done
</commit_message>
<xml_diff>
--- a/results/monthly_returns.xlsx
+++ b/results/monthly_returns.xlsx
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,24 +45,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -435,453 +421,453 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>VW</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>MVP</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="1" t="n">
         <v>41670</v>
       </c>
       <c r="B2" t="n">
         <v>-0.03577051251348723</v>
       </c>
       <c r="C2" t="n">
-        <v>2.730222653296241e-06</v>
+        <v>2.730222653150524e-06</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="1" t="n">
         <v>41698</v>
       </c>
       <c r="B3" t="n">
         <v>0.05457272646088732</v>
       </c>
       <c r="C3" t="n">
-        <v>0.04891788266058272</v>
+        <v>0.04891788266058264</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="1" t="n">
         <v>41729</v>
       </c>
       <c r="B4" t="n">
         <v>0.007762261335563271</v>
       </c>
       <c r="C4" t="n">
-        <v>0.002976221230969092</v>
+        <v>0.00297622123096899</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="1" t="n">
         <v>41759</v>
       </c>
       <c r="B5" t="n">
         <v>0.01583202208543277</v>
       </c>
       <c r="C5" t="n">
-        <v>0.01963062223914375</v>
+        <v>0.01963062223914377</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="1" t="n">
         <v>41789</v>
       </c>
       <c r="B6" t="n">
         <v>0.01643020929599076</v>
       </c>
       <c r="C6" t="n">
-        <v>0.007681447610686079</v>
+        <v>0.007681447610686071</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="1" t="n">
         <v>41820</v>
       </c>
       <c r="B7" t="n">
         <v>0.01148059602195001</v>
       </c>
       <c r="C7" t="n">
-        <v>0.005367108850342378</v>
+        <v>0.005367108850342425</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="1" t="n">
         <v>41851</v>
       </c>
       <c r="B8" t="n">
         <v>-0.023164508181366</v>
       </c>
       <c r="C8" t="n">
-        <v>-0.04029218519291357</v>
+        <v>-0.04029218519291371</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="1" t="n">
         <v>41880</v>
       </c>
       <c r="B9" t="n">
         <v>0.02457691833184666</v>
       </c>
       <c r="C9" t="n">
-        <v>0.02976601488670122</v>
+        <v>0.02976601488670137</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="1" t="n">
         <v>41912</v>
       </c>
       <c r="B10" t="n">
         <v>-0.02330935776278098</v>
       </c>
       <c r="C10" t="n">
-        <v>-0.03905226153597566</v>
+        <v>-0.0390522615359757</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="1" t="n">
         <v>41943</v>
       </c>
       <c r="B11" t="n">
         <v>0.004941866289649032</v>
       </c>
       <c r="C11" t="n">
-        <v>0.04655124954081642</v>
+        <v>0.04655124954081648</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="1" t="n">
         <v>41971</v>
       </c>
       <c r="B12" t="n">
         <v>0.02684646801091424</v>
       </c>
       <c r="C12" t="n">
-        <v>0.03060666196916687</v>
+        <v>0.03060666196916704</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="1" t="n">
         <v>42004</v>
       </c>
       <c r="B13" t="n">
         <v>-0.01793837814404243</v>
       </c>
       <c r="C13" t="n">
-        <v>0.005229028925359638</v>
+        <v>0.005229028925359563</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="1" t="n">
         <v>42034</v>
       </c>
       <c r="B14" t="n">
         <v>-0.02282175733578628</v>
       </c>
       <c r="C14" t="n">
-        <v>0.003962826851777302</v>
+        <v>0.003962826851777556</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n">
+      <c r="A15" s="1" t="n">
         <v>42062</v>
       </c>
       <c r="B15" t="n">
         <v>0.05685610170123574</v>
       </c>
       <c r="C15" t="n">
-        <v>0.003828721582178348</v>
+        <v>0.00382872158217545</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
+      <c r="A16" s="1" t="n">
         <v>42094</v>
       </c>
       <c r="B16" t="n">
         <v>-0.01878225285036577</v>
       </c>
       <c r="C16" t="n">
-        <v>-0.01384128158689765</v>
+        <v>-0.01384128158688789</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n">
+      <c r="A17" s="1" t="n">
         <v>42124</v>
       </c>
       <c r="B17" t="n">
         <v>0.02217672013381462</v>
       </c>
       <c r="C17" t="n">
-        <v>0.00249267189554782</v>
+        <v>0.002492671895549026</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n">
+      <c r="A18" s="1" t="n">
         <v>42153</v>
       </c>
       <c r="B18" t="n">
         <v>0.002763819717271396</v>
       </c>
       <c r="C18" t="n">
-        <v>0.01117211679002529</v>
+        <v>0.01117211679003133</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n">
+      <c r="A19" s="1" t="n">
         <v>42185</v>
       </c>
       <c r="B19" t="n">
         <v>-0.02380750565336756</v>
       </c>
       <c r="C19" t="n">
-        <v>-0.02617371908367839</v>
+        <v>-0.02617371908367149</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
+      <c r="A20" s="1" t="n">
         <v>42216</v>
       </c>
       <c r="B20" t="n">
         <v>0.01953878974553074</v>
       </c>
       <c r="C20" t="n">
-        <v>0.04865401254988987</v>
+        <v>0.04865401254992193</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n">
+      <c r="A21" s="1" t="n">
         <v>42247</v>
       </c>
       <c r="B21" t="n">
         <v>-0.06371876922900283</v>
       </c>
       <c r="C21" t="n">
-        <v>-0.03001587259349209</v>
+        <v>-0.03001587259348153</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n">
+      <c r="A22" s="1" t="n">
         <v>42277</v>
       </c>
       <c r="B22" t="n">
         <v>-0.03029360394779007</v>
       </c>
       <c r="C22" t="n">
-        <v>-0.01279551909589483</v>
+        <v>-0.0127955190958921</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n">
+      <c r="A23" s="1" t="n">
         <v>42307</v>
       </c>
       <c r="B23" t="n">
         <v>0.07484781831623569</v>
       </c>
       <c r="C23" t="n">
-        <v>0.02227678680400481</v>
+        <v>0.02227678680398361</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n">
+      <c r="A24" s="1" t="n">
         <v>42338</v>
       </c>
       <c r="B24" t="n">
         <v>-0.005311215995536839</v>
       </c>
       <c r="C24" t="n">
-        <v>-0.006476912681978852</v>
+        <v>-0.006476912681995494</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n">
+      <c r="A25" s="1" t="n">
         <v>42369</v>
       </c>
       <c r="B25" t="n">
         <v>-0.02288379535149846</v>
       </c>
       <c r="C25" t="n">
-        <v>0.02650813033797008</v>
+        <v>0.02650813033797372</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n">
+      <c r="A26" s="1" t="n">
         <v>42398</v>
       </c>
       <c r="B26" t="n">
         <v>-0.05258465528398181</v>
       </c>
       <c r="C26" t="n">
-        <v>0.007202263417535389</v>
+        <v>0.007202263417544447</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="n">
+      <c r="A27" s="1" t="n">
         <v>42429</v>
       </c>
       <c r="B27" t="n">
         <v>-0.008168481738206232</v>
       </c>
       <c r="C27" t="n">
-        <v>-0.004129525619331957</v>
+        <v>-0.004129525619341459</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n">
+      <c r="A28" s="1" t="n">
         <v>42460</v>
       </c>
       <c r="B28" t="n">
         <v>0.07050360052854185</v>
       </c>
       <c r="C28" t="n">
-        <v>0.04860880597789544</v>
+        <v>0.04860880597788868</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n">
+      <c r="A29" s="1" t="n">
         <v>42489</v>
       </c>
       <c r="B29" t="n">
         <v>0.01346581614572162</v>
       </c>
       <c r="C29" t="n">
-        <v>0.01856700237040006</v>
+        <v>0.01856700237040105</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n">
+      <c r="A30" s="1" t="n">
         <v>42521</v>
       </c>
       <c r="B30" t="n">
         <v>0.00659258352088357</v>
       </c>
       <c r="C30" t="n">
-        <v>0.01027099558763584</v>
+        <v>0.01027099558763282</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n">
+      <c r="A31" s="1" t="n">
         <v>42551</v>
       </c>
       <c r="B31" t="n">
         <v>-0.01362076122737209</v>
       </c>
       <c r="C31" t="n">
-        <v>0.05701160541280054</v>
+        <v>0.0570116054128005</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n">
+      <c r="A32" s="1" t="n">
         <v>42580</v>
       </c>
       <c r="B32" t="n">
         <v>0.03674407370358323</v>
       </c>
       <c r="C32" t="n">
-        <v>0.02028425692060203</v>
+        <v>0.02028425692059983</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n">
+      <c r="A33" s="1" t="n">
         <v>42613</v>
       </c>
       <c r="B33" t="n">
         <v>0.002077100500778767</v>
       </c>
       <c r="C33" t="n">
-        <v>-0.04585631771577894</v>
+        <v>-0.04585631771578419</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n">
+      <c r="A34" s="1" t="n">
         <v>42643</v>
       </c>
       <c r="B34" t="n">
         <v>0.002306627011404471</v>
       </c>
       <c r="C34" t="n">
-        <v>-0.01514616317556969</v>
+        <v>-0.01514616317556679</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="n">
+      <c r="A35" s="1" t="n">
         <v>42674</v>
       </c>
       <c r="B35" t="n">
         <v>-0.02102440381119557</v>
       </c>
       <c r="C35" t="n">
-        <v>-0.03581039563151144</v>
+        <v>-0.03581039563152387</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n">
+      <c r="A36" s="1" t="n">
         <v>42704</v>
       </c>
       <c r="B36" t="n">
         <v>0.01819181100066963</v>
       </c>
       <c r="C36" t="n">
-        <v>-0.0203794617939423</v>
+        <v>-0.02037946179393673</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n">
+      <c r="A37" s="1" t="n">
         <v>42734</v>
       </c>
       <c r="B37" t="n">
         <v>0.03324819018946118</v>
       </c>
       <c r="C37" t="n">
-        <v>0.02901604237318184</v>
+        <v>0.02901604237318179</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n">
+      <c r="A38" s="1" t="n">
         <v>42766</v>
       </c>
       <c r="B38" t="n">
         <v>0.01579079678590857</v>
       </c>
       <c r="C38" t="n">
-        <v>0.008000296440244407</v>
+        <v>0.008000296440244394</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="n">
+      <c r="A39" s="1" t="n">
         <v>42794</v>
       </c>
       <c r="B39" t="n">
         <v>0.02844322118409615</v>
       </c>
       <c r="C39" t="n">
-        <v>0.02103760038850297</v>
+        <v>0.02103760038850296</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n">
+      <c r="A40" s="1" t="n">
         <v>42825</v>
       </c>
       <c r="B40" t="n">
         <v>0.01407803634341376</v>
       </c>
       <c r="C40" t="n">
-        <v>0.003774695669464323</v>
+        <v>0.003774695669464308</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="n">
+      <c r="A41" s="1" t="n">
         <v>42853</v>
       </c>
       <c r="B41" t="n">
@@ -892,293 +878,293 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n">
+      <c r="A42" s="1" t="n">
         <v>42886</v>
       </c>
       <c r="B42" t="n">
         <v>0.02654951259123661</v>
       </c>
       <c r="C42" t="n">
-        <v>0.03242084510237631</v>
+        <v>0.03242084510237632</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="n">
+      <c r="A43" s="1" t="n">
         <v>42916</v>
       </c>
       <c r="B43" t="n">
         <v>0.002373678903860118</v>
       </c>
       <c r="C43" t="n">
-        <v>-0.01179985612409164</v>
+        <v>-0.01179985612409165</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n">
+      <c r="A44" s="1" t="n">
         <v>42947</v>
       </c>
       <c r="B44" t="n">
         <v>0.02246463779799775</v>
       </c>
       <c r="C44" t="n">
-        <v>0.02283386439866803</v>
+        <v>0.02283386439866797</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n">
+      <c r="A45" s="1" t="n">
         <v>42978</v>
       </c>
       <c r="B45" t="n">
         <v>0.00244198517741814</v>
       </c>
       <c r="C45" t="n">
-        <v>-0.04791840198244816</v>
+        <v>-0.04791840198244822</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n">
+      <c r="A46" s="1" t="n">
         <v>43007</v>
       </c>
       <c r="B46" t="n">
         <v>0.02808540905124245</v>
       </c>
       <c r="C46" t="n">
-        <v>0.008226210958247351</v>
+        <v>0.008226210958247446</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="n">
+      <c r="A47" s="1" t="n">
         <v>43039</v>
       </c>
       <c r="B47" t="n">
         <v>0.01894898151901998</v>
       </c>
       <c r="C47" t="n">
-        <v>0.01965537009971235</v>
+        <v>0.01965537009971226</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="n">
+      <c r="A48" s="1" t="n">
         <v>43069</v>
       </c>
       <c r="B48" t="n">
         <v>0.02194443635302347</v>
       </c>
       <c r="C48" t="n">
-        <v>0.03785084198989316</v>
+        <v>0.03785084198989323</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="n">
+      <c r="A49" s="1" t="n">
         <v>43098</v>
       </c>
       <c r="B49" t="n">
         <v>0.01303863736857334</v>
       </c>
       <c r="C49" t="n">
-        <v>0.02080060156683981</v>
+        <v>0.02080060156683984</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="n">
+      <c r="A50" s="1" t="n">
         <v>43131</v>
       </c>
       <c r="B50" t="n">
         <v>0.04951854951058408</v>
       </c>
       <c r="C50" t="n">
-        <v>-0.02108269564772554</v>
+        <v>-0.02108269564772578</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="n">
+      <c r="A51" s="1" t="n">
         <v>43159</v>
       </c>
       <c r="B51" t="n">
         <v>-0.04705500135027535</v>
       </c>
       <c r="C51" t="n">
-        <v>-0.07538499118428517</v>
+        <v>-0.07538499118428529</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="n">
+      <c r="A52" s="1" t="n">
         <v>43189</v>
       </c>
       <c r="B52" t="n">
         <v>-0.01795301847933335</v>
       </c>
       <c r="C52" t="n">
-        <v>-0.006770242963501999</v>
+        <v>-0.006770242963501949</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="n">
+      <c r="A53" s="1" t="n">
         <v>43220</v>
       </c>
       <c r="B53" t="n">
         <v>0.01261748230660959</v>
       </c>
       <c r="C53" t="n">
-        <v>0.0103740841945414</v>
+        <v>0.01037408419454142</v>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="n">
+      <c r="A54" s="1" t="n">
         <v>43251</v>
       </c>
       <c r="B54" t="n">
         <v>0.001351174902387803</v>
       </c>
       <c r="C54" t="n">
-        <v>0.0008495935373884897</v>
+        <v>0.0008495935373884849</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="n">
+      <c r="A55" s="1" t="n">
         <v>43280</v>
       </c>
       <c r="B55" t="n">
         <v>0.0002616030988843816</v>
       </c>
       <c r="C55" t="n">
-        <v>0.01688277897535898</v>
+        <v>0.01688277897535887</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="n">
+      <c r="A56" s="1" t="n">
         <v>43312</v>
       </c>
       <c r="B56" t="n">
         <v>0.03849477634390881</v>
       </c>
       <c r="C56" t="n">
-        <v>0.007820125985214546</v>
+        <v>0.007820125985214475</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="n">
+      <c r="A57" s="1" t="n">
         <v>43343</v>
       </c>
       <c r="B57" t="n">
         <v>0.008992745924063218</v>
       </c>
       <c r="C57" t="n">
-        <v>0.03077127343045237</v>
+        <v>0.03077127343045231</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="n">
+      <c r="A58" s="1" t="n">
         <v>43371</v>
       </c>
       <c r="B58" t="n">
         <v>0.0066165392530823</v>
       </c>
       <c r="C58" t="n">
-        <v>-0.006763939976214333</v>
+        <v>-0.006763939976214378</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="n">
+      <c r="A59" s="1" t="n">
         <v>43404</v>
       </c>
       <c r="B59" t="n">
         <v>-0.06453623148170358</v>
       </c>
       <c r="C59" t="n">
-        <v>-0.008528733589575378</v>
+        <v>-0.008528733589575333</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="n">
+      <c r="A60" s="1" t="n">
         <v>43434</v>
       </c>
       <c r="B60" t="n">
         <v>0.01111789623001095</v>
       </c>
       <c r="C60" t="n">
-        <v>-0.02543711892555225</v>
+        <v>-0.02543711892555279</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="n">
+      <c r="A61" s="1" t="n">
         <v>43465</v>
       </c>
       <c r="B61" t="n">
         <v>-0.07816398564554208</v>
       </c>
       <c r="C61" t="n">
-        <v>-0.06309782624436877</v>
+        <v>-0.06309782624436892</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="n">
+      <c r="A62" s="1" t="n">
         <v>43496</v>
       </c>
       <c r="B62" t="n">
         <v>0.07601880736345278</v>
       </c>
       <c r="C62" t="n">
-        <v>0.01825868070332333</v>
+        <v>0.01825868070332343</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="n">
+      <c r="A63" s="1" t="n">
         <v>43524</v>
       </c>
       <c r="B63" t="n">
         <v>0.03326236662472595</v>
       </c>
       <c r="C63" t="n">
-        <v>0.03715013667570122</v>
+        <v>0.03715013667570118</v>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="n">
+      <c r="A64" s="1" t="n">
         <v>43553</v>
       </c>
       <c r="B64" t="n">
         <v>0.01472293864230933</v>
       </c>
       <c r="C64" t="n">
-        <v>0.03795096554228373</v>
+        <v>0.0379509655422837</v>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="n">
+      <c r="A65" s="1" t="n">
         <v>43585</v>
       </c>
       <c r="B65" t="n">
         <v>0.03766175186714266</v>
       </c>
       <c r="C65" t="n">
-        <v>0.03182501970714726</v>
+        <v>0.03182501970714718</v>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="n">
+      <c r="A66" s="1" t="n">
         <v>43616</v>
       </c>
       <c r="B66" t="n">
         <v>-0.06023474533191252</v>
       </c>
       <c r="C66" t="n">
-        <v>-0.01913396723817573</v>
+        <v>-0.01913396723817571</v>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="n">
+      <c r="A67" s="1" t="n">
         <v>43644</v>
       </c>
       <c r="B67" t="n">
         <v>0.07033903461068169</v>
       </c>
       <c r="C67" t="n">
-        <v>0.03889138671042749</v>
+        <v>0.03889138671042734</v>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="n">
+      <c r="A68" s="1" t="n">
         <v>43677</v>
       </c>
       <c r="B68" t="n">
@@ -1189,227 +1175,227 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="n">
+      <c r="A69" s="1" t="n">
         <v>43707</v>
       </c>
       <c r="B69" t="n">
         <v>-0.01828779657461423</v>
       </c>
       <c r="C69" t="n">
-        <v>0.00614656552630522</v>
+        <v>0.006146565526305313</v>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="n">
+      <c r="A70" s="1" t="n">
         <v>43738</v>
       </c>
       <c r="B70" t="n">
         <v>0.02466315429160364</v>
       </c>
       <c r="C70" t="n">
-        <v>0.01044742051010836</v>
+        <v>0.01044742051010839</v>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="n">
+      <c r="A71" s="1" t="n">
         <v>43769</v>
       </c>
       <c r="B71" t="n">
         <v>0.02217750538357088</v>
       </c>
       <c r="C71" t="n">
-        <v>-0.005609037583084878</v>
+        <v>-0.005609037583084731</v>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="n">
+      <c r="A72" s="1" t="n">
         <v>43798</v>
       </c>
       <c r="B72" t="n">
         <v>0.02997799889267743</v>
       </c>
       <c r="C72" t="n">
-        <v>0.01917680945616541</v>
+        <v>0.01917680945616537</v>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="n">
+      <c r="A73" s="1" t="n">
         <v>43830</v>
       </c>
       <c r="B73" t="n">
         <v>0.03482421028928007</v>
       </c>
       <c r="C73" t="n">
-        <v>0.04255413156749994</v>
+        <v>0.04255413156750001</v>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="n">
+      <c r="A74" s="1" t="n">
         <v>43861</v>
       </c>
       <c r="B74" t="n">
         <v>-0.009580265949088524</v>
       </c>
       <c r="C74" t="n">
-        <v>0.01409299279690879</v>
+        <v>0.0140929927969088</v>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="n">
+      <c r="A75" s="1" t="n">
         <v>43889</v>
       </c>
       <c r="B75" t="n">
         <v>-0.08791498768503248</v>
       </c>
       <c r="C75" t="n">
-        <v>-0.08525920946399368</v>
+        <v>-0.08525920946399373</v>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="n">
+      <c r="A76" s="1" t="n">
         <v>43921</v>
       </c>
       <c r="B76" t="n">
         <v>-0.1306650921429244</v>
       </c>
       <c r="C76" t="n">
-        <v>-0.1247491258960358</v>
+        <v>-0.124749125896036</v>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="n">
+      <c r="A77" s="1" t="n">
         <v>43951</v>
       </c>
       <c r="B77" t="n">
         <v>0.1075112783889687</v>
       </c>
       <c r="C77" t="n">
-        <v>0.1110485181262049</v>
+        <v>0.111048518126205</v>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="n">
+      <c r="A78" s="1" t="n">
         <v>43980</v>
       </c>
       <c r="B78" t="n">
         <v>0.04142078875265022</v>
       </c>
       <c r="C78" t="n">
-        <v>0.02457496452175814</v>
+        <v>0.02457496452175811</v>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="n">
+      <c r="A79" s="1" t="n">
         <v>44012</v>
       </c>
       <c r="B79" t="n">
         <v>0.02854315181783309</v>
       </c>
       <c r="C79" t="n">
-        <v>-0.009407842664746651</v>
+        <v>-0.009407842664746665</v>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="n">
+      <c r="A80" s="1" t="n">
         <v>44043</v>
       </c>
       <c r="B80" t="n">
         <v>0.04883592322798035</v>
       </c>
       <c r="C80" t="n">
-        <v>0.07388733025686642</v>
+        <v>0.07388733025686636</v>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="2" t="n">
+      <c r="A81" s="1" t="n">
         <v>44074</v>
       </c>
       <c r="B81" t="n">
         <v>0.06540930795489953</v>
       </c>
       <c r="C81" t="n">
-        <v>0.03472996518892831</v>
+        <v>0.0347299651889283</v>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="n">
+      <c r="A82" s="1" t="n">
         <v>44104</v>
       </c>
       <c r="B82" t="n">
         <v>-0.03798082063905267</v>
       </c>
       <c r="C82" t="n">
-        <v>-0.01828587876157301</v>
+        <v>-0.01828587876157299</v>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="2" t="n">
+      <c r="A83" s="1" t="n">
         <v>44134</v>
       </c>
       <c r="B83" t="n">
         <v>-0.03589474696672947</v>
       </c>
       <c r="C83" t="n">
-        <v>-0.01852884685448301</v>
+        <v>-0.018528846854483</v>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="n">
+      <c r="A84" s="1" t="n">
         <v>44165</v>
       </c>
       <c r="B84" t="n">
         <v>0.1283940181539289</v>
       </c>
       <c r="C84" t="n">
-        <v>0.07337263320928981</v>
+        <v>0.07337263320928987</v>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="n">
+      <c r="A85" s="1" t="n">
         <v>44196</v>
       </c>
       <c r="B85" t="n">
         <v>0.03983956548531003</v>
       </c>
       <c r="C85" t="n">
-        <v>0.02761180067773917</v>
+        <v>0.02761180067773927</v>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="n">
+      <c r="A86" s="1" t="n">
         <v>44225</v>
       </c>
       <c r="B86" t="n">
         <v>-0.01212400733186289</v>
       </c>
       <c r="C86" t="n">
-        <v>-0.00847554794687993</v>
+        <v>-0.008475547946880116</v>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="2" t="n">
+      <c r="A87" s="1" t="n">
         <v>44253</v>
       </c>
       <c r="B87" t="n">
         <v>0.02733062300679211</v>
       </c>
       <c r="C87" t="n">
-        <v>-0.0002929385122206005</v>
+        <v>-0.0002929385122203247</v>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="2" t="n">
+      <c r="A88" s="1" t="n">
         <v>44286</v>
       </c>
       <c r="B88" t="n">
         <v>0.04536283607748608</v>
       </c>
       <c r="C88" t="n">
-        <v>0.07860679864833139</v>
+        <v>0.07860679864833137</v>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="2" t="n">
+      <c r="A89" s="1" t="n">
         <v>44316</v>
       </c>
       <c r="B89" t="n">
@@ -1420,62 +1406,62 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="n">
+      <c r="A90" s="1" t="n">
         <v>44347</v>
       </c>
       <c r="B90" t="n">
         <v>0.02015621412882964</v>
       </c>
       <c r="C90" t="n">
-        <v>0.02586177073086892</v>
+        <v>0.02586177073086889</v>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="2" t="n">
+      <c r="A91" s="1" t="n">
         <v>44377</v>
       </c>
       <c r="B91" t="n">
         <v>0.009085467039068967</v>
       </c>
       <c r="C91" t="n">
-        <v>-0.02045945211371527</v>
+        <v>-0.0204594521137154</v>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="2" t="n">
+      <c r="A92" s="1" t="n">
         <v>44407</v>
       </c>
       <c r="B92" t="n">
         <v>0.01882876021698834</v>
       </c>
       <c r="C92" t="n">
-        <v>0.02666338376474659</v>
+        <v>0.02666338376474656</v>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="2" t="n">
+      <c r="A93" s="1" t="n">
         <v>44439</v>
       </c>
       <c r="B93" t="n">
         <v>0.02292599245632672</v>
       </c>
       <c r="C93" t="n">
-        <v>0.002387439376513896</v>
+        <v>0.002387439376513915</v>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="2" t="n">
+      <c r="A94" s="1" t="n">
         <v>44469</v>
       </c>
       <c r="B94" t="n">
         <v>-0.04484438196599666</v>
       </c>
       <c r="C94" t="n">
-        <v>-0.06122936085079826</v>
+        <v>-0.06122936085079829</v>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="2" t="n">
+      <c r="A95" s="1" t="n">
         <v>44498</v>
       </c>
       <c r="B95" t="n">
@@ -1486,205 +1472,205 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="2" t="n">
+      <c r="A96" s="1" t="n">
         <v>44530</v>
       </c>
       <c r="B96" t="n">
         <v>-0.01485364644369896</v>
       </c>
       <c r="C96" t="n">
-        <v>-0.03396186432802809</v>
+        <v>-0.03396186432802805</v>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="2" t="n">
+      <c r="A97" s="1" t="n">
         <v>44561</v>
       </c>
       <c r="B97" t="n">
         <v>0.05275242494481132</v>
       </c>
       <c r="C97" t="n">
-        <v>0.07491379473672655</v>
+        <v>0.07491379473672632</v>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="2" t="n">
+      <c r="A98" s="1" t="n">
         <v>44592</v>
       </c>
       <c r="B98" t="n">
         <v>-0.04101565747775374</v>
       </c>
       <c r="C98" t="n">
-        <v>-0.01040777410931704</v>
+        <v>-0.01040777410931138</v>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="2" t="n">
+      <c r="A99" s="1" t="n">
         <v>44620</v>
       </c>
       <c r="B99" t="n">
         <v>-0.02440661653703706</v>
       </c>
       <c r="C99" t="n">
-        <v>-0.0186504067041853</v>
+        <v>-0.0186504067041889</v>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="2" t="n">
+      <c r="A100" s="1" t="n">
         <v>44651</v>
       </c>
       <c r="B100" t="n">
         <v>0.02739841992527333</v>
       </c>
       <c r="C100" t="n">
-        <v>0.04370183673260929</v>
+        <v>0.04370183673260911</v>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="2" t="n">
+      <c r="A101" s="1" t="n">
         <v>44680</v>
       </c>
       <c r="B101" t="n">
         <v>-0.07246087523648355</v>
       </c>
       <c r="C101" t="n">
-        <v>-0.02808252545282783</v>
+        <v>-0.02808252545283147</v>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="2" t="n">
+      <c r="A102" s="1" t="n">
         <v>44712</v>
       </c>
       <c r="B102" t="n">
         <v>0.005871650263511217</v>
       </c>
       <c r="C102" t="n">
-        <v>0.0102332581273923</v>
+        <v>0.01023325812738706</v>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="2" t="n">
+      <c r="A103" s="1" t="n">
         <v>44742</v>
       </c>
       <c r="B103" t="n">
         <v>-0.08596805176643892</v>
       </c>
       <c r="C103" t="n">
-        <v>-0.05379045931733725</v>
+        <v>-0.05379045931736158</v>
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="2" t="n">
+      <c r="A104" s="1" t="n">
         <v>44771</v>
       </c>
       <c r="B104" t="n">
         <v>0.07919681433848735</v>
       </c>
       <c r="C104" t="n">
-        <v>0.02639147983836548</v>
+        <v>0.02639147983837267</v>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="2" t="n">
+      <c r="A105" s="1" t="n">
         <v>44804</v>
       </c>
       <c r="B105" t="n">
         <v>-0.04332771130830771</v>
       </c>
       <c r="C105" t="n">
-        <v>-0.03353423439714249</v>
+        <v>-0.03353423439715109</v>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="2" t="n">
+      <c r="A106" s="1" t="n">
         <v>44834</v>
       </c>
       <c r="B106" t="n">
         <v>-0.09169976227284632</v>
       </c>
       <c r="C106" t="n">
-        <v>-0.08064395506676628</v>
+        <v>-0.08064395506674363</v>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="2" t="n">
+      <c r="A107" s="1" t="n">
         <v>44865</v>
       </c>
       <c r="B107" t="n">
         <v>0.08600326884212639</v>
       </c>
       <c r="C107" t="n">
-        <v>0.06432684165012396</v>
+        <v>0.06432684165014646</v>
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="2" t="n">
+      <c r="A108" s="1" t="n">
         <v>44895</v>
       </c>
       <c r="B108" t="n">
         <v>0.07019817439074505</v>
       </c>
       <c r="C108" t="n">
-        <v>0.05811044115168718</v>
+        <v>0.05811044115169554</v>
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="2" t="n">
+      <c r="A109" s="1" t="n">
         <v>44925</v>
       </c>
       <c r="B109" t="n">
         <v>-0.04196388752670809</v>
       </c>
       <c r="C109" t="n">
-        <v>-0.02738915085564868</v>
+        <v>-0.02738915085563594</v>
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="2" t="n">
+      <c r="A110" s="1" t="n">
         <v>44957</v>
       </c>
       <c r="B110" t="n">
         <v>0.06616089743523371</v>
       </c>
       <c r="C110" t="n">
-        <v>0.02469967352489337</v>
+        <v>0.02469967352489349</v>
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="2" t="n">
+      <c r="A111" s="1" t="n">
         <v>44985</v>
       </c>
       <c r="B111" t="n">
         <v>-0.02239431803222399</v>
       </c>
       <c r="C111" t="n">
-        <v>-0.002891586717282327</v>
+        <v>-0.00289158671728222</v>
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="2" t="n">
+      <c r="A112" s="1" t="n">
         <v>45016</v>
       </c>
       <c r="B112" t="n">
         <v>0.03122580989791321</v>
       </c>
       <c r="C112" t="n">
-        <v>0.01357216473408997</v>
+        <v>0.01357216473408979</v>
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="2" t="n">
+      <c r="A113" s="1" t="n">
         <v>45044</v>
       </c>
       <c r="B113" t="n">
         <v>0.02644255003476621</v>
       </c>
       <c r="C113" t="n">
-        <v>0.0266580687084309</v>
+        <v>0.02665806870843073</v>
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="2" t="n">
+      <c r="A114" s="1" t="n">
         <v>45077</v>
       </c>
       <c r="B114" t="n">
@@ -1695,238 +1681,238 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="2" t="n">
+      <c r="A115" s="1" t="n">
         <v>45107</v>
       </c>
       <c r="B115" t="n">
         <v>0.06093188600225954</v>
       </c>
       <c r="C115" t="n">
-        <v>0.01356101307124181</v>
+        <v>0.01356101307124157</v>
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="2" t="n">
+      <c r="A116" s="1" t="n">
         <v>45138</v>
       </c>
       <c r="B116" t="n">
         <v>0.0290835962367811</v>
       </c>
       <c r="C116" t="n">
-        <v>0.007779183779411563</v>
+        <v>0.007779183779411554</v>
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="2" t="n">
+      <c r="A117" s="1" t="n">
         <v>45169</v>
       </c>
       <c r="B117" t="n">
         <v>-0.02253641802697804</v>
       </c>
       <c r="C117" t="n">
-        <v>-0.01816153083576296</v>
+        <v>-0.01816153083576303</v>
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="2" t="n">
+      <c r="A118" s="1" t="n">
         <v>45198</v>
       </c>
       <c r="B118" t="n">
         <v>-0.04645542708300802</v>
       </c>
       <c r="C118" t="n">
-        <v>-0.0469587878042293</v>
+        <v>-0.04695878780422914</v>
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="2" t="n">
+      <c r="A119" s="1" t="n">
         <v>45230</v>
       </c>
       <c r="B119" t="n">
         <v>-0.02171054624420314</v>
       </c>
       <c r="C119" t="n">
-        <v>-0.007236148857404119</v>
+        <v>-0.007236148857404152</v>
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="2" t="n">
+      <c r="A120" s="1" t="n">
         <v>45260</v>
       </c>
       <c r="B120" t="n">
         <v>0.09051414707262974</v>
       </c>
       <c r="C120" t="n">
-        <v>0.02714817936583044</v>
+        <v>0.02714817936583027</v>
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="2" t="n">
+      <c r="A121" s="1" t="n">
         <v>45289</v>
       </c>
       <c r="B121" t="n">
         <v>0.04513240680873794</v>
       </c>
       <c r="C121" t="n">
-        <v>0.01303706415322593</v>
+        <v>0.01303706415322584</v>
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="2" t="n">
+      <c r="A122" s="1" t="n">
         <v>45322</v>
       </c>
       <c r="B122" t="n">
         <v>0.01245418746238778</v>
       </c>
       <c r="C122" t="n">
-        <v>-0.009093756460092309</v>
+        <v>-0.009093756460089478</v>
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="2" t="n">
+      <c r="A123" s="1" t="n">
         <v>45351</v>
       </c>
       <c r="B123" t="n">
         <v>0.03901825082531514</v>
       </c>
       <c r="C123" t="n">
-        <v>0.03594891098855772</v>
+        <v>0.0359489109885649</v>
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="2" t="n">
+      <c r="A124" s="1" t="n">
         <v>45380</v>
       </c>
       <c r="B124" t="n">
         <v>0.03637442820614256</v>
       </c>
       <c r="C124" t="n">
-        <v>0.02523437034638649</v>
+        <v>0.02523437034638502</v>
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="2" t="n">
+      <c r="A125" s="1" t="n">
         <v>45412</v>
       </c>
       <c r="B125" t="n">
         <v>-0.03609511822437324</v>
       </c>
       <c r="C125" t="n">
-        <v>0.01904789933259306</v>
+        <v>0.019047899332591</v>
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="2" t="n">
+      <c r="A126" s="1" t="n">
         <v>45443</v>
       </c>
       <c r="B126" t="n">
         <v>0.05159895294222033</v>
       </c>
       <c r="C126" t="n">
-        <v>0.02202757570791832</v>
+        <v>0.02202757570791411</v>
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="2" t="n">
+      <c r="A127" s="1" t="n">
         <v>45471</v>
       </c>
       <c r="B127" t="n">
         <v>0.01673400189527829</v>
       </c>
       <c r="C127" t="n">
-        <v>-0.01700788360701016</v>
+        <v>-0.01700788360700735</v>
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="2" t="n">
+      <c r="A128" s="1" t="n">
         <v>45504</v>
       </c>
       <c r="B128" t="n">
         <v>0.01638886236175519</v>
       </c>
       <c r="C128" t="n">
-        <v>0.02504571085099221</v>
+        <v>0.02504571085099025</v>
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="2" t="n">
+      <c r="A129" s="1" t="n">
         <v>45534</v>
       </c>
       <c r="B129" t="n">
         <v>0.02662711852757172</v>
       </c>
       <c r="C129" t="n">
-        <v>0.03280900611413946</v>
+        <v>0.03280900611414459</v>
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="2" t="n">
+      <c r="A130" s="1" t="n">
         <v>45565</v>
       </c>
       <c r="B130" t="n">
         <v>0.01491367792089069</v>
       </c>
       <c r="C130" t="n">
-        <v>-0.005177790269040606</v>
+        <v>-0.005177790269040688</v>
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="2" t="n">
+      <c r="A131" s="1" t="n">
         <v>45596</v>
       </c>
       <c r="B131" t="n">
         <v>-0.02230215658726872</v>
       </c>
       <c r="C131" t="n">
-        <v>-0.0444944105699025</v>
+        <v>-0.0444944105699073</v>
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="2" t="n">
+      <c r="A132" s="1" t="n">
         <v>45625</v>
       </c>
       <c r="B132" t="n">
         <v>0.04154212052715963</v>
       </c>
       <c r="C132" t="n">
-        <v>-0.006102921933923455</v>
+        <v>-0.006102921933921876</v>
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="2" t="n">
+      <c r="A133" s="1" t="n">
         <v>45657</v>
       </c>
       <c r="B133" t="n">
         <v>-0.03216767101109499</v>
       </c>
       <c r="C133" t="n">
-        <v>-0.02658561534534758</v>
+        <v>-0.02658561534534414</v>
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="2" t="n">
+      <c r="A134" s="1" t="n">
         <v>45688</v>
       </c>
       <c r="B134" t="n">
         <v>0.03074400383563204</v>
       </c>
       <c r="C134" t="n">
-        <v>-0.006027115472455938</v>
+        <v>-0.006027115472455921</v>
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="2" t="n">
+      <c r="A135" s="1" t="n">
         <v>45716</v>
       </c>
       <c r="B135" t="n">
         <v>0.005356171982461908</v>
       </c>
       <c r="C135" t="n">
-        <v>0.00530682315910169</v>
+        <v>0.005306823159101683</v>
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="2" t="n">
+      <c r="A136" s="1" t="n">
         <v>45747</v>
       </c>
       <c r="B136" t="n">
@@ -1937,102 +1923,102 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="2" t="n">
+      <c r="A137" s="1" t="n">
         <v>45777</v>
       </c>
       <c r="B137" t="n">
         <v>-0.0003712512432697251</v>
       </c>
       <c r="C137" t="n">
-        <v>0.04393901351277295</v>
+        <v>0.04393901351277293</v>
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="2" t="n">
+      <c r="A138" s="1" t="n">
         <v>45807</v>
       </c>
       <c r="B138" t="n">
         <v>0.05049871444190139</v>
       </c>
       <c r="C138" t="n">
-        <v>-0.01871251790217802</v>
+        <v>-0.01871251790217808</v>
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="2" t="n">
+      <c r="A139" s="1" t="n">
         <v>45838</v>
       </c>
       <c r="B139" t="n">
         <v>0.043684099601013</v>
       </c>
       <c r="C139" t="n">
-        <v>-0.00703258854949062</v>
+        <v>-0.007032588549490621</v>
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="2" t="n">
+      <c r="A140" s="1" t="n">
         <v>45869</v>
       </c>
       <c r="B140" t="n">
         <v>0.01704349688554993</v>
       </c>
       <c r="C140" t="n">
-        <v>-0.003793539940815127</v>
+        <v>-0.003793539940815096</v>
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="2" t="n">
+      <c r="A141" s="1" t="n">
         <v>45898</v>
       </c>
       <c r="B141" t="n">
         <v>0.02376419689285764</v>
       </c>
       <c r="C141" t="n">
-        <v>0.009855526705872236</v>
+        <v>0.009855526705872263</v>
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="2" t="n">
+      <c r="A142" s="1" t="n">
         <v>45930</v>
       </c>
       <c r="B142" t="n">
         <v>0.02752594267972975</v>
       </c>
       <c r="C142" t="n">
-        <v>0.004432415254182237</v>
+        <v>0.004432415254182327</v>
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="2" t="n">
+      <c r="A143" s="1" t="n">
         <v>45961</v>
       </c>
       <c r="B143" t="n">
         <v>0.02345311271306457</v>
       </c>
       <c r="C143" t="n">
-        <v>-0.0150512307646178</v>
+        <v>-0.01505123076461782</v>
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="2" t="n">
+      <c r="A144" s="1" t="n">
         <v>45989</v>
       </c>
       <c r="B144" t="n">
         <v>0.007211569097595304</v>
       </c>
       <c r="C144" t="n">
-        <v>0.05424916396365363</v>
+        <v>0.05424916396365365</v>
       </c>
     </row>
     <row r="145">
-      <c r="A145" s="2" t="n">
+      <c r="A145" s="1" t="n">
         <v>46022</v>
       </c>
       <c r="B145" t="n">
         <v>0.0145794998106231</v>
       </c>
       <c r="C145" t="n">
-        <v>0.003868600951347357</v>
+        <v>0.00386860095134728</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Test Single Factor + Ledoit
</commit_message>
<xml_diff>
--- a/results/monthly_returns.xlsx
+++ b/results/monthly_returns.xlsx
@@ -20,13 +20,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,13 +48,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -421,1604 +435,1604 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>VW</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>MVP</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" s="2" t="n">
         <v>41670</v>
       </c>
       <c r="B2" t="n">
         <v>-0.03577051251348723</v>
       </c>
       <c r="C2" t="n">
-        <v>2.730222653150524e-06</v>
+        <v>-0.00481655169826153</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" s="2" t="n">
         <v>41698</v>
       </c>
       <c r="B3" t="n">
         <v>0.05457272646088732</v>
       </c>
       <c r="C3" t="n">
-        <v>0.04891788266058264</v>
+        <v>0.04729606898759194</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" s="2" t="n">
         <v>41729</v>
       </c>
       <c r="B4" t="n">
         <v>0.007762261335563271</v>
       </c>
       <c r="C4" t="n">
-        <v>0.00297622123096899</v>
+        <v>0.006338661632828502</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" s="2" t="n">
         <v>41759</v>
       </c>
       <c r="B5" t="n">
         <v>0.01583202208543277</v>
       </c>
       <c r="C5" t="n">
-        <v>0.01963062223914377</v>
+        <v>0.02011146048383985</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" s="2" t="n">
         <v>41789</v>
       </c>
       <c r="B6" t="n">
         <v>0.01643020929599076</v>
       </c>
       <c r="C6" t="n">
-        <v>0.007681447610686071</v>
+        <v>0.007680340939861655</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" s="2" t="n">
         <v>41820</v>
       </c>
       <c r="B7" t="n">
         <v>0.01148059602195001</v>
       </c>
       <c r="C7" t="n">
-        <v>0.005367108850342425</v>
+        <v>0.006578384151253187</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" s="2" t="n">
         <v>41851</v>
       </c>
       <c r="B8" t="n">
         <v>-0.023164508181366</v>
       </c>
       <c r="C8" t="n">
-        <v>-0.04029218519291371</v>
+        <v>-0.04172244099755235</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" s="2" t="n">
         <v>41880</v>
       </c>
       <c r="B9" t="n">
         <v>0.02457691833184666</v>
       </c>
       <c r="C9" t="n">
-        <v>0.02976601488670137</v>
+        <v>0.03003256291393353</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" s="2" t="n">
         <v>41912</v>
       </c>
       <c r="B10" t="n">
         <v>-0.02330935776278098</v>
       </c>
       <c r="C10" t="n">
-        <v>-0.03905226153597569</v>
+        <v>-0.03777058560841617</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" s="2" t="n">
         <v>41943</v>
       </c>
       <c r="B11" t="n">
         <v>0.004941866289649032</v>
       </c>
       <c r="C11" t="n">
-        <v>0.04655124954081647</v>
+        <v>0.04772787202912362</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" s="2" t="n">
         <v>41971</v>
       </c>
       <c r="B12" t="n">
         <v>0.02684646801091424</v>
       </c>
       <c r="C12" t="n">
-        <v>0.03060666196916705</v>
+        <v>0.02867714961939459</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" s="2" t="n">
         <v>42004</v>
       </c>
       <c r="B13" t="n">
         <v>-0.01793837814404243</v>
       </c>
       <c r="C13" t="n">
-        <v>0.005229028925359567</v>
+        <v>0.005606131058487454</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" s="2" t="n">
         <v>42034</v>
       </c>
       <c r="B14" t="n">
         <v>-0.02282175733578628</v>
       </c>
       <c r="C14" t="n">
-        <v>0.003962826851777557</v>
+        <v>0.003664408129007701</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" s="2" t="n">
         <v>42062</v>
       </c>
       <c r="B15" t="n">
         <v>0.05685610170123574</v>
       </c>
       <c r="C15" t="n">
-        <v>0.00382872158217545</v>
+        <v>0.0103595629767555</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" s="2" t="n">
         <v>42094</v>
       </c>
       <c r="B16" t="n">
         <v>-0.01878225285036577</v>
       </c>
       <c r="C16" t="n">
-        <v>-0.01384128158688788</v>
+        <v>-0.01551358338958826</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
+      <c r="A17" s="2" t="n">
         <v>42124</v>
       </c>
       <c r="B17" t="n">
         <v>0.02217672013381462</v>
       </c>
       <c r="C17" t="n">
-        <v>0.002492671895549026</v>
+        <v>0.003728819189570185</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
+      <c r="A18" s="2" t="n">
         <v>42153</v>
       </c>
       <c r="B18" t="n">
         <v>0.002763819717271396</v>
       </c>
       <c r="C18" t="n">
-        <v>0.01117211679003133</v>
+        <v>0.01141952297075848</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
+      <c r="A19" s="2" t="n">
         <v>42185</v>
       </c>
       <c r="B19" t="n">
         <v>-0.02380750565336756</v>
       </c>
       <c r="C19" t="n">
-        <v>-0.02617371908367149</v>
+        <v>-0.02379966753639999</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
+      <c r="A20" s="2" t="n">
         <v>42216</v>
       </c>
       <c r="B20" t="n">
         <v>0.01953878974553074</v>
       </c>
       <c r="C20" t="n">
-        <v>0.04865401254992193</v>
+        <v>0.04705376305557753</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
+      <c r="A21" s="2" t="n">
         <v>42247</v>
       </c>
       <c r="B21" t="n">
         <v>-0.06371876922900283</v>
       </c>
       <c r="C21" t="n">
-        <v>-0.03001587259348153</v>
+        <v>-0.03222375860079314</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
+      <c r="A22" s="2" t="n">
         <v>42277</v>
       </c>
       <c r="B22" t="n">
         <v>-0.03029360394779007</v>
       </c>
       <c r="C22" t="n">
-        <v>-0.0127955190958921</v>
+        <v>-0.008770416705412308</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
+      <c r="A23" s="2" t="n">
         <v>42307</v>
       </c>
       <c r="B23" t="n">
         <v>0.07484781831623569</v>
       </c>
       <c r="C23" t="n">
-        <v>0.02227678680398361</v>
+        <v>0.03254103088179028</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
+      <c r="A24" s="2" t="n">
         <v>42338</v>
       </c>
       <c r="B24" t="n">
         <v>-0.005311215995536839</v>
       </c>
       <c r="C24" t="n">
-        <v>-0.006476912681995494</v>
+        <v>-0.004947861051835726</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
+      <c r="A25" s="2" t="n">
         <v>42369</v>
       </c>
       <c r="B25" t="n">
         <v>-0.02288379535149846</v>
       </c>
       <c r="C25" t="n">
-        <v>0.02650813033797373</v>
+        <v>0.021924486432785</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
+      <c r="A26" s="2" t="n">
         <v>42398</v>
       </c>
       <c r="B26" t="n">
         <v>-0.05258465528398181</v>
       </c>
       <c r="C26" t="n">
-        <v>0.007202263417544444</v>
+        <v>0.007974664155795813</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
+      <c r="A27" s="2" t="n">
         <v>42429</v>
       </c>
       <c r="B27" t="n">
         <v>-0.008168481738206232</v>
       </c>
       <c r="C27" t="n">
-        <v>-0.004129525619341459</v>
+        <v>-0.003837105733913564</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
+      <c r="A28" s="2" t="n">
         <v>42460</v>
       </c>
       <c r="B28" t="n">
         <v>0.07050360052854185</v>
       </c>
       <c r="C28" t="n">
-        <v>0.0486088059778887</v>
+        <v>0.04918728092849432</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
+      <c r="A29" s="2" t="n">
         <v>42489</v>
       </c>
       <c r="B29" t="n">
         <v>0.01346581614572162</v>
       </c>
       <c r="C29" t="n">
-        <v>0.01856700237040105</v>
+        <v>0.01755568581401722</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="n">
+      <c r="A30" s="2" t="n">
         <v>42521</v>
       </c>
       <c r="B30" t="n">
         <v>0.00659258352088357</v>
       </c>
       <c r="C30" t="n">
-        <v>0.01027099558763282</v>
+        <v>0.01093559364503575</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="n">
+      <c r="A31" s="2" t="n">
         <v>42551</v>
       </c>
       <c r="B31" t="n">
         <v>-0.01362076122737209</v>
       </c>
       <c r="C31" t="n">
-        <v>0.0570116054128005</v>
+        <v>0.04948549266523025</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="n">
+      <c r="A32" s="2" t="n">
         <v>42580</v>
       </c>
       <c r="B32" t="n">
         <v>0.03674407370358323</v>
       </c>
       <c r="C32" t="n">
-        <v>0.02028425692059982</v>
+        <v>0.01751486591933996</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="n">
+      <c r="A33" s="2" t="n">
         <v>42613</v>
       </c>
       <c r="B33" t="n">
         <v>0.002077100500778767</v>
       </c>
       <c r="C33" t="n">
-        <v>-0.0458563177157842</v>
+        <v>-0.04435458387739791</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="n">
+      <c r="A34" s="2" t="n">
         <v>42643</v>
       </c>
       <c r="B34" t="n">
         <v>0.002306627011404471</v>
       </c>
       <c r="C34" t="n">
-        <v>-0.01514617636029168</v>
+        <v>-0.01263750947580846</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="n">
+      <c r="A35" s="2" t="n">
         <v>42674</v>
       </c>
       <c r="B35" t="n">
         <v>-0.02102440381119557</v>
       </c>
       <c r="C35" t="n">
-        <v>-0.03581042728386113</v>
+        <v>-0.03559367844640302</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="n">
+      <c r="A36" s="2" t="n">
         <v>42704</v>
       </c>
       <c r="B36" t="n">
         <v>0.01819181100066963</v>
       </c>
       <c r="C36" t="n">
-        <v>-0.02037946179393672</v>
+        <v>-0.01657266317125299</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="n">
+      <c r="A37" s="2" t="n">
         <v>42734</v>
       </c>
       <c r="B37" t="n">
         <v>0.03324819018946118</v>
       </c>
       <c r="C37" t="n">
-        <v>0.02901606558443876</v>
+        <v>0.03049639813702271</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="n">
+      <c r="A38" s="2" t="n">
         <v>42766</v>
       </c>
       <c r="B38" t="n">
         <v>0.01579079678590857</v>
       </c>
       <c r="C38" t="n">
-        <v>0.008000296440244394</v>
+        <v>0.01269401296900648</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n">
+      <c r="A39" s="2" t="n">
         <v>42794</v>
       </c>
       <c r="B39" t="n">
         <v>0.02844322118409615</v>
       </c>
       <c r="C39" t="n">
-        <v>0.02103760038850296</v>
+        <v>0.01727109970099426</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="n">
+      <c r="A40" s="2" t="n">
         <v>42825</v>
       </c>
       <c r="B40" t="n">
         <v>0.01407803634341376</v>
       </c>
       <c r="C40" t="n">
-        <v>0.003774695669464308</v>
+        <v>0.005368514886413911</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="n">
+      <c r="A41" s="2" t="n">
         <v>42853</v>
       </c>
       <c r="B41" t="n">
         <v>0.01822042462107884</v>
       </c>
       <c r="C41" t="n">
-        <v>0.03669626479655809</v>
+        <v>0.03372608753678873</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="n">
+      <c r="A42" s="2" t="n">
         <v>42886</v>
       </c>
       <c r="B42" t="n">
         <v>0.02654951259123661</v>
       </c>
       <c r="C42" t="n">
-        <v>0.03242084510237632</v>
+        <v>0.02447867586817949</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="n">
+      <c r="A43" s="2" t="n">
         <v>42916</v>
       </c>
       <c r="B43" t="n">
         <v>0.002373678903860118</v>
       </c>
       <c r="C43" t="n">
-        <v>-0.01179985612409165</v>
+        <v>-0.01489892288061603</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="n">
+      <c r="A44" s="2" t="n">
         <v>42947</v>
       </c>
       <c r="B44" t="n">
         <v>0.02246463779799775</v>
       </c>
       <c r="C44" t="n">
-        <v>0.02283386439866797</v>
+        <v>0.01620659347711604</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="n">
+      <c r="A45" s="2" t="n">
         <v>42978</v>
       </c>
       <c r="B45" t="n">
         <v>0.00244198517741814</v>
       </c>
       <c r="C45" t="n">
-        <v>-0.04791840198244822</v>
+        <v>-0.04122869241558448</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="n">
+      <c r="A46" s="2" t="n">
         <v>43007</v>
       </c>
       <c r="B46" t="n">
         <v>0.02808540905124245</v>
       </c>
       <c r="C46" t="n">
-        <v>0.008226210958247446</v>
+        <v>0.006177166231987881</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="n">
+      <c r="A47" s="2" t="n">
         <v>43039</v>
       </c>
       <c r="B47" t="n">
         <v>0.01894898151901998</v>
       </c>
       <c r="C47" t="n">
-        <v>0.01965537009971226</v>
+        <v>0.01337724871896624</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="n">
+      <c r="A48" s="2" t="n">
         <v>43069</v>
       </c>
       <c r="B48" t="n">
         <v>0.02194443635302347</v>
       </c>
       <c r="C48" t="n">
-        <v>0.03785084198989323</v>
+        <v>0.02517856070949299</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1" t="n">
+      <c r="A49" s="2" t="n">
         <v>43098</v>
       </c>
       <c r="B49" t="n">
         <v>0.01303863736857334</v>
       </c>
       <c r="C49" t="n">
-        <v>0.02080060156683984</v>
+        <v>0.01561468135456912</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1" t="n">
+      <c r="A50" s="2" t="n">
         <v>43131</v>
       </c>
       <c r="B50" t="n">
         <v>0.04951854951058408</v>
       </c>
       <c r="C50" t="n">
-        <v>-0.02108269564772578</v>
+        <v>-0.01684920269582513</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="n">
+      <c r="A51" s="2" t="n">
         <v>43159</v>
       </c>
       <c r="B51" t="n">
         <v>-0.04705500135027535</v>
       </c>
       <c r="C51" t="n">
-        <v>-0.07538499118428529</v>
+        <v>-0.06616802133795754</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1" t="n">
+      <c r="A52" s="2" t="n">
         <v>43189</v>
       </c>
       <c r="B52" t="n">
         <v>-0.01795301847933335</v>
       </c>
       <c r="C52" t="n">
-        <v>-0.006770242963501949</v>
+        <v>-0.008152559113326623</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="1" t="n">
+      <c r="A53" s="2" t="n">
         <v>43220</v>
       </c>
       <c r="B53" t="n">
         <v>0.01261748230660959</v>
       </c>
       <c r="C53" t="n">
-        <v>0.01037408419454142</v>
+        <v>0.008830318043337011</v>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="1" t="n">
+      <c r="A54" s="2" t="n">
         <v>43251</v>
       </c>
       <c r="B54" t="n">
         <v>0.001351174902387803</v>
       </c>
       <c r="C54" t="n">
-        <v>0.0008495935373884849</v>
+        <v>0.01104551890546974</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="n">
+      <c r="A55" s="2" t="n">
         <v>43280</v>
       </c>
       <c r="B55" t="n">
         <v>0.0002616030988843816</v>
       </c>
       <c r="C55" t="n">
-        <v>0.01688277897535887</v>
+        <v>0.02090510194355684</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="1" t="n">
+      <c r="A56" s="2" t="n">
         <v>43312</v>
       </c>
       <c r="B56" t="n">
         <v>0.03849477634390881</v>
       </c>
       <c r="C56" t="n">
-        <v>0.007820125985214475</v>
+        <v>0.01051489736295047</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="1" t="n">
+      <c r="A57" s="2" t="n">
         <v>43343</v>
       </c>
       <c r="B57" t="n">
         <v>0.008992745924063218</v>
       </c>
       <c r="C57" t="n">
-        <v>0.03077127343045231</v>
+        <v>0.0208282511001946</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="1" t="n">
+      <c r="A58" s="2" t="n">
         <v>43371</v>
       </c>
       <c r="B58" t="n">
         <v>0.0066165392530823</v>
       </c>
       <c r="C58" t="n">
-        <v>-0.006763939976214378</v>
+        <v>-0.005263103626727206</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="1" t="n">
+      <c r="A59" s="2" t="n">
         <v>43404</v>
       </c>
       <c r="B59" t="n">
         <v>-0.06453623148170358</v>
       </c>
       <c r="C59" t="n">
-        <v>-0.008528733589575333</v>
+        <v>-0.01818643607555086</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="1" t="n">
+      <c r="A60" s="2" t="n">
         <v>43434</v>
       </c>
       <c r="B60" t="n">
         <v>0.01111789623001095</v>
       </c>
       <c r="C60" t="n">
-        <v>-0.02543711892555279</v>
+        <v>-0.003706219951176296</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="1" t="n">
+      <c r="A61" s="2" t="n">
         <v>43465</v>
       </c>
       <c r="B61" t="n">
         <v>-0.07816398564554208</v>
       </c>
       <c r="C61" t="n">
-        <v>-0.06309782624436892</v>
+        <v>-0.06307783494331633</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="1" t="n">
+      <c r="A62" s="2" t="n">
         <v>43496</v>
       </c>
       <c r="B62" t="n">
         <v>0.07601880736345278</v>
       </c>
       <c r="C62" t="n">
-        <v>0.01825868070332343</v>
+        <v>0.02063107719080389</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="1" t="n">
+      <c r="A63" s="2" t="n">
         <v>43524</v>
       </c>
       <c r="B63" t="n">
         <v>0.03326236662472595</v>
       </c>
       <c r="C63" t="n">
-        <v>0.03715013667570118</v>
+        <v>0.03825593402676782</v>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="1" t="n">
+      <c r="A64" s="2" t="n">
         <v>43553</v>
       </c>
       <c r="B64" t="n">
         <v>0.01472293864230933</v>
       </c>
       <c r="C64" t="n">
-        <v>0.0379509655422837</v>
+        <v>0.03494084912618512</v>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="1" t="n">
+      <c r="A65" s="2" t="n">
         <v>43585</v>
       </c>
       <c r="B65" t="n">
         <v>0.03766175186714266</v>
       </c>
       <c r="C65" t="n">
-        <v>0.03182501970714718</v>
+        <v>0.02737376576035037</v>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="1" t="n">
+      <c r="A66" s="2" t="n">
         <v>43616</v>
       </c>
       <c r="B66" t="n">
         <v>-0.06023474533191252</v>
       </c>
       <c r="C66" t="n">
-        <v>-0.0191339672381757</v>
+        <v>-0.02222157984850629</v>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="1" t="n">
+      <c r="A67" s="2" t="n">
         <v>43644</v>
       </c>
       <c r="B67" t="n">
         <v>0.07033903461068169</v>
       </c>
       <c r="C67" t="n">
-        <v>0.03889138671042734</v>
+        <v>0.04186613772142073</v>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="1" t="n">
+      <c r="A68" s="2" t="n">
         <v>43677</v>
       </c>
       <c r="B68" t="n">
         <v>0.00439947754685985</v>
       </c>
       <c r="C68" t="n">
-        <v>0.01163044013186628</v>
+        <v>0.009522815551679513</v>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="1" t="n">
+      <c r="A69" s="2" t="n">
         <v>43707</v>
       </c>
       <c r="B69" t="n">
         <v>-0.01828779657461423</v>
       </c>
       <c r="C69" t="n">
-        <v>0.006146565526305315</v>
+        <v>0.0152103331585349</v>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="1" t="n">
+      <c r="A70" s="2" t="n">
         <v>43738</v>
       </c>
       <c r="B70" t="n">
         <v>0.02466315429160364</v>
       </c>
       <c r="C70" t="n">
-        <v>0.01044742051010839</v>
+        <v>0.006604812653261417</v>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="1" t="n">
+      <c r="A71" s="2" t="n">
         <v>43769</v>
       </c>
       <c r="B71" t="n">
         <v>0.02217750538357088</v>
       </c>
       <c r="C71" t="n">
-        <v>-0.005609037583084736</v>
+        <v>-0.001327221783458397</v>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="1" t="n">
+      <c r="A72" s="2" t="n">
         <v>43798</v>
       </c>
       <c r="B72" t="n">
         <v>0.02997799889267743</v>
       </c>
       <c r="C72" t="n">
-        <v>0.01917680945616537</v>
+        <v>0.01873125958053234</v>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="1" t="n">
+      <c r="A73" s="2" t="n">
         <v>43830</v>
       </c>
       <c r="B73" t="n">
         <v>0.03482421028928007</v>
       </c>
       <c r="C73" t="n">
-        <v>0.0425541315675</v>
+        <v>0.04193944098221207</v>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="1" t="n">
+      <c r="A74" s="2" t="n">
         <v>43861</v>
       </c>
       <c r="B74" t="n">
         <v>-0.009580265949088524</v>
       </c>
       <c r="C74" t="n">
-        <v>0.0140929927969088</v>
+        <v>0.01169955204495742</v>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="1" t="n">
+      <c r="A75" s="2" t="n">
         <v>43889</v>
       </c>
       <c r="B75" t="n">
         <v>-0.08791498768503248</v>
       </c>
       <c r="C75" t="n">
-        <v>-0.08525920946399373</v>
+        <v>-0.08547222154564432</v>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="1" t="n">
+      <c r="A76" s="2" t="n">
         <v>43921</v>
       </c>
       <c r="B76" t="n">
         <v>-0.1306650921429244</v>
       </c>
       <c r="C76" t="n">
-        <v>-0.124749125896036</v>
+        <v>-0.1177459164809954</v>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="1" t="n">
+      <c r="A77" s="2" t="n">
         <v>43951</v>
       </c>
       <c r="B77" t="n">
         <v>0.1075112783889687</v>
       </c>
       <c r="C77" t="n">
-        <v>0.1110485181262049</v>
+        <v>0.107370588150448</v>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="1" t="n">
+      <c r="A78" s="2" t="n">
         <v>43980</v>
       </c>
       <c r="B78" t="n">
         <v>0.04142078875265022</v>
       </c>
       <c r="C78" t="n">
-        <v>0.02457496452175811</v>
+        <v>0.0261562079345386</v>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="1" t="n">
+      <c r="A79" s="2" t="n">
         <v>44012</v>
       </c>
       <c r="B79" t="n">
         <v>0.02854315181783309</v>
       </c>
       <c r="C79" t="n">
-        <v>-0.009407842664746665</v>
+        <v>-0.01060515899879751</v>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="1" t="n">
+      <c r="A80" s="2" t="n">
         <v>44043</v>
       </c>
       <c r="B80" t="n">
         <v>0.04883592322798035</v>
       </c>
       <c r="C80" t="n">
-        <v>0.07388733025686639</v>
+        <v>0.07148084680712641</v>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="1" t="n">
+      <c r="A81" s="2" t="n">
         <v>44074</v>
       </c>
       <c r="B81" t="n">
         <v>0.06540930795489953</v>
       </c>
       <c r="C81" t="n">
-        <v>0.0347299651889283</v>
+        <v>0.03204056865028183</v>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="1" t="n">
+      <c r="A82" s="2" t="n">
         <v>44104</v>
       </c>
       <c r="B82" t="n">
         <v>-0.03798082063905267</v>
       </c>
       <c r="C82" t="n">
-        <v>-0.01828587876157299</v>
+        <v>-0.01792825628676786</v>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="1" t="n">
+      <c r="A83" s="2" t="n">
         <v>44134</v>
       </c>
       <c r="B83" t="n">
         <v>-0.03589474696672947</v>
       </c>
       <c r="C83" t="n">
-        <v>-0.018528846854483</v>
+        <v>-0.01878108115765808</v>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="1" t="n">
+      <c r="A84" s="2" t="n">
         <v>44165</v>
       </c>
       <c r="B84" t="n">
         <v>0.1283940181539289</v>
       </c>
       <c r="C84" t="n">
-        <v>0.07337263320928987</v>
+        <v>0.07259584873826545</v>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="1" t="n">
+      <c r="A85" s="2" t="n">
         <v>44196</v>
       </c>
       <c r="B85" t="n">
         <v>0.03983956548531003</v>
       </c>
       <c r="C85" t="n">
-        <v>0.02761180067773927</v>
+        <v>0.0289022890468589</v>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="1" t="n">
+      <c r="A86" s="2" t="n">
         <v>44225</v>
       </c>
       <c r="B86" t="n">
         <v>-0.01212400733186289</v>
       </c>
       <c r="C86" t="n">
-        <v>-0.008475547946880119</v>
+        <v>-0.005245280012396868</v>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="1" t="n">
+      <c r="A87" s="2" t="n">
         <v>44253</v>
       </c>
       <c r="B87" t="n">
         <v>0.02733062300679211</v>
       </c>
       <c r="C87" t="n">
-        <v>-0.0002929385122203247</v>
+        <v>-0.004572640806403129</v>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="1" t="n">
+      <c r="A88" s="2" t="n">
         <v>44286</v>
       </c>
       <c r="B88" t="n">
         <v>0.04536283607748608</v>
       </c>
       <c r="C88" t="n">
-        <v>0.07860679864833137</v>
+        <v>0.08262019648589847</v>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="1" t="n">
+      <c r="A89" s="2" t="n">
         <v>44316</v>
       </c>
       <c r="B89" t="n">
         <v>0.05016847426313767</v>
       </c>
       <c r="C89" t="n">
-        <v>0.02201364011522929</v>
+        <v>0.02432179160466919</v>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="1" t="n">
+      <c r="A90" s="2" t="n">
         <v>44347</v>
       </c>
       <c r="B90" t="n">
         <v>0.02015621412882964</v>
       </c>
       <c r="C90" t="n">
-        <v>0.02586177073086889</v>
+        <v>0.02393516928225115</v>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="1" t="n">
+      <c r="A91" s="2" t="n">
         <v>44377</v>
       </c>
       <c r="B91" t="n">
         <v>0.009085467039068967</v>
       </c>
       <c r="C91" t="n">
-        <v>-0.0204594521137154</v>
+        <v>-0.01672115604024303</v>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="1" t="n">
+      <c r="A92" s="2" t="n">
         <v>44407</v>
       </c>
       <c r="B92" t="n">
         <v>0.01882876021698834</v>
       </c>
       <c r="C92" t="n">
-        <v>0.02666338376474656</v>
+        <v>0.02842117726803394</v>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="1" t="n">
+      <c r="A93" s="2" t="n">
         <v>44439</v>
       </c>
       <c r="B93" t="n">
         <v>0.02292599245632672</v>
       </c>
       <c r="C93" t="n">
-        <v>0.002387439376513915</v>
+        <v>0.007994830845347073</v>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="1" t="n">
+      <c r="A94" s="2" t="n">
         <v>44469</v>
       </c>
       <c r="B94" t="n">
         <v>-0.04484438196599666</v>
       </c>
       <c r="C94" t="n">
-        <v>-0.06122936085079829</v>
+        <v>-0.05847634547353054</v>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="1" t="n">
+      <c r="A95" s="2" t="n">
         <v>44498</v>
       </c>
       <c r="B95" t="n">
         <v>0.06369195815598885</v>
       </c>
       <c r="C95" t="n">
-        <v>0.03782405411565329</v>
+        <v>0.03517308509824792</v>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="1" t="n">
+      <c r="A96" s="2" t="n">
         <v>44530</v>
       </c>
       <c r="B96" t="n">
         <v>-0.01485364644369896</v>
       </c>
       <c r="C96" t="n">
-        <v>-0.03396186432802804</v>
+        <v>-0.03091858192901106</v>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="1" t="n">
+      <c r="A97" s="2" t="n">
         <v>44561</v>
       </c>
       <c r="B97" t="n">
         <v>0.05275242494481132</v>
       </c>
       <c r="C97" t="n">
-        <v>0.07491379473672632</v>
+        <v>0.08029981468635675</v>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="1" t="n">
+      <c r="A98" s="2" t="n">
         <v>44592</v>
       </c>
       <c r="B98" t="n">
         <v>-0.04101565747775374</v>
       </c>
       <c r="C98" t="n">
-        <v>-0.0107165330128023</v>
+        <v>-0.01778649764724247</v>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="1" t="n">
+      <c r="A99" s="2" t="n">
         <v>44620</v>
       </c>
       <c r="B99" t="n">
         <v>-0.02440661653703706</v>
       </c>
       <c r="C99" t="n">
-        <v>-0.01920971128139254</v>
+        <v>-0.01232212651185563</v>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="1" t="n">
+      <c r="A100" s="2" t="n">
         <v>44651</v>
       </c>
       <c r="B100" t="n">
         <v>0.02739841992527333</v>
       </c>
       <c r="C100" t="n">
-        <v>0.04503775512071487</v>
+        <v>0.04908304111674888</v>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="1" t="n">
+      <c r="A101" s="2" t="n">
         <v>44680</v>
       </c>
       <c r="B101" t="n">
         <v>-0.07246087523648355</v>
       </c>
       <c r="C101" t="n">
-        <v>-0.02890403427392126</v>
+        <v>-0.03172862178691287</v>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="1" t="n">
+      <c r="A102" s="2" t="n">
         <v>44712</v>
       </c>
       <c r="B102" t="n">
         <v>0.005871650263511217</v>
       </c>
       <c r="C102" t="n">
-        <v>0.01054152570454194</v>
+        <v>0.01051186310250954</v>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="1" t="n">
+      <c r="A103" s="2" t="n">
         <v>44742</v>
       </c>
       <c r="B103" t="n">
         <v>-0.08596805176643892</v>
       </c>
       <c r="C103" t="n">
-        <v>-0.05539453431691729</v>
+        <v>-0.05507990205327662</v>
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="1" t="n">
+      <c r="A104" s="2" t="n">
         <v>44771</v>
       </c>
       <c r="B104" t="n">
         <v>0.07919681433848735</v>
       </c>
       <c r="C104" t="n">
-        <v>0.02722464807773119</v>
+        <v>0.03604613722076366</v>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="1" t="n">
+      <c r="A105" s="2" t="n">
         <v>44804</v>
       </c>
       <c r="B105" t="n">
         <v>-0.04332771130830771</v>
       </c>
       <c r="C105" t="n">
-        <v>-0.03456547844680725</v>
+        <v>-0.02626497467782272</v>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="1" t="n">
+      <c r="A106" s="2" t="n">
         <v>44834</v>
       </c>
       <c r="B106" t="n">
         <v>-0.09169976227284632</v>
       </c>
       <c r="C106" t="n">
-        <v>-0.08321347390671704</v>
+        <v>-0.08290421413523899</v>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="1" t="n">
+      <c r="A107" s="2" t="n">
         <v>44865</v>
       </c>
       <c r="B107" t="n">
         <v>0.08600326884212639</v>
       </c>
       <c r="C107" t="n">
-        <v>0.06656374022556116</v>
+        <v>0.06998622899605189</v>
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="1" t="n">
+      <c r="A108" s="2" t="n">
         <v>44895</v>
       </c>
       <c r="B108" t="n">
         <v>0.07019817439074505</v>
       </c>
       <c r="C108" t="n">
-        <v>0.06000589040282032</v>
+        <v>0.05977169149329654</v>
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="1" t="n">
+      <c r="A109" s="2" t="n">
         <v>44925</v>
       </c>
       <c r="B109" t="n">
         <v>-0.04196388752670809</v>
       </c>
       <c r="C109" t="n">
-        <v>-0.0282320851797198</v>
+        <v>-0.02823064212783596</v>
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="1" t="n">
+      <c r="A110" s="2" t="n">
         <v>44957</v>
       </c>
       <c r="B110" t="n">
         <v>0.06616089743523371</v>
       </c>
       <c r="C110" t="n">
-        <v>0.02474933607455884</v>
+        <v>0.02393514447393397</v>
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="1" t="n">
+      <c r="A111" s="2" t="n">
         <v>44985</v>
       </c>
       <c r="B111" t="n">
         <v>-0.02239431803222399</v>
       </c>
       <c r="C111" t="n">
-        <v>-0.002897260286726776</v>
+        <v>-0.006891280812889752</v>
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="1" t="n">
+      <c r="A112" s="2" t="n">
         <v>45016</v>
       </c>
       <c r="B112" t="n">
         <v>0.03122580989791321</v>
       </c>
       <c r="C112" t="n">
-        <v>0.01359887199607428</v>
+        <v>0.0118421415057038</v>
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="1" t="n">
+      <c r="A113" s="2" t="n">
         <v>45044</v>
       </c>
       <c r="B113" t="n">
         <v>0.02644255003476621</v>
       </c>
       <c r="C113" t="n">
-        <v>0.02670985760782062</v>
+        <v>0.02734082497437937</v>
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="1" t="n">
+      <c r="A114" s="2" t="n">
         <v>45077</v>
       </c>
       <c r="B114" t="n">
         <v>-0.01825027086054789</v>
       </c>
       <c r="C114" t="n">
-        <v>-0.04502583939860093</v>
+        <v>-0.04681455207830134</v>
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="1" t="n">
+      <c r="A115" s="2" t="n">
         <v>45107</v>
       </c>
       <c r="B115" t="n">
         <v>0.06093188600225954</v>
       </c>
       <c r="C115" t="n">
-        <v>0.01407704306086305</v>
+        <v>0.01631181051322894</v>
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="1" t="n">
+      <c r="A116" s="2" t="n">
         <v>45138</v>
       </c>
       <c r="B116" t="n">
         <v>0.0290835962367811</v>
       </c>
       <c r="C116" t="n">
-        <v>0.008071099605955883</v>
+        <v>0.008283814823725661</v>
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="1" t="n">
+      <c r="A117" s="2" t="n">
         <v>45169</v>
       </c>
       <c r="B117" t="n">
         <v>-0.02253641802697804</v>
       </c>
       <c r="C117" t="n">
-        <v>-0.01883759037941291</v>
+        <v>-0.02450943501530416</v>
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="1" t="n">
+      <c r="A118" s="2" t="n">
         <v>45198</v>
       </c>
       <c r="B118" t="n">
         <v>-0.04645542708300802</v>
       </c>
       <c r="C118" t="n">
-        <v>-0.04874041055883954</v>
+        <v>-0.04398133864991243</v>
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="1" t="n">
+      <c r="A119" s="2" t="n">
         <v>45230</v>
       </c>
       <c r="B119" t="n">
         <v>-0.02171054624420314</v>
       </c>
       <c r="C119" t="n">
-        <v>-0.007524767532574535</v>
+        <v>-0.01101723542670296</v>
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="1" t="n">
+      <c r="A120" s="2" t="n">
         <v>45260</v>
       </c>
       <c r="B120" t="n">
         <v>0.09051414707262974</v>
       </c>
       <c r="C120" t="n">
-        <v>0.02823921257206482</v>
+        <v>0.03459969159971101</v>
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="1" t="n">
+      <c r="A121" s="2" t="n">
         <v>45289</v>
       </c>
       <c r="B121" t="n">
         <v>0.04513240680873794</v>
       </c>
       <c r="C121" t="n">
-        <v>0.01354665298453042</v>
+        <v>0.01908374117738183</v>
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="1" t="n">
+      <c r="A122" s="2" t="n">
         <v>45322</v>
       </c>
       <c r="B122" t="n">
         <v>0.01245418746238778</v>
       </c>
       <c r="C122" t="n">
-        <v>-0.009093756460089475</v>
+        <v>-0.002972561984548144</v>
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="1" t="n">
+      <c r="A123" s="2" t="n">
         <v>45351</v>
       </c>
       <c r="B123" t="n">
         <v>0.03901825082531514</v>
       </c>
       <c r="C123" t="n">
-        <v>0.0359489109885649</v>
+        <v>0.02182263764553104</v>
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="1" t="n">
+      <c r="A124" s="2" t="n">
         <v>45380</v>
       </c>
       <c r="B124" t="n">
         <v>0.03637442820614256</v>
       </c>
       <c r="C124" t="n">
-        <v>0.02523437034638502</v>
+        <v>0.02766588670083584</v>
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="1" t="n">
+      <c r="A125" s="2" t="n">
         <v>45412</v>
       </c>
       <c r="B125" t="n">
         <v>-0.03609511822437324</v>
       </c>
       <c r="C125" t="n">
-        <v>0.019047899332591</v>
+        <v>0.007887485409802872</v>
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="1" t="n">
+      <c r="A126" s="2" t="n">
         <v>45443</v>
       </c>
       <c r="B126" t="n">
         <v>0.05159895294222033</v>
       </c>
       <c r="C126" t="n">
-        <v>0.02202757570791411</v>
+        <v>0.03008781794761481</v>
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="1" t="n">
+      <c r="A127" s="2" t="n">
         <v>45471</v>
       </c>
       <c r="B127" t="n">
         <v>0.01673400189527829</v>
       </c>
       <c r="C127" t="n">
-        <v>-0.01700788360700735</v>
+        <v>-0.01003117137510173</v>
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="1" t="n">
+      <c r="A128" s="2" t="n">
         <v>45504</v>
       </c>
       <c r="B128" t="n">
         <v>0.01638886236175519</v>
       </c>
       <c r="C128" t="n">
-        <v>0.02504571085099026</v>
+        <v>0.0273998663907862</v>
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="1" t="n">
+      <c r="A129" s="2" t="n">
         <v>45534</v>
       </c>
       <c r="B129" t="n">
         <v>0.02662711852757172</v>
       </c>
       <c r="C129" t="n">
-        <v>0.03280900611414458</v>
+        <v>0.04480272094453801</v>
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="1" t="n">
+      <c r="A130" s="2" t="n">
         <v>45565</v>
       </c>
       <c r="B130" t="n">
         <v>0.01491367792089069</v>
       </c>
       <c r="C130" t="n">
-        <v>-0.005177790269040686</v>
+        <v>-0.005980811556354734</v>
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="1" t="n">
+      <c r="A131" s="2" t="n">
         <v>45596</v>
       </c>
       <c r="B131" t="n">
         <v>-0.02230215658726872</v>
       </c>
       <c r="C131" t="n">
-        <v>-0.0444944105699073</v>
+        <v>-0.04647168819412067</v>
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="1" t="n">
+      <c r="A132" s="2" t="n">
         <v>45625</v>
       </c>
       <c r="B132" t="n">
         <v>0.04154212052715963</v>
       </c>
       <c r="C132" t="n">
-        <v>-0.006102921933921878</v>
+        <v>-6.588281982651892e-05</v>
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="1" t="n">
+      <c r="A133" s="2" t="n">
         <v>45657</v>
       </c>
       <c r="B133" t="n">
         <v>-0.03216767101109499</v>
       </c>
       <c r="C133" t="n">
-        <v>-0.02658561534534414</v>
+        <v>-0.03434676809823738</v>
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="1" t="n">
+      <c r="A134" s="2" t="n">
         <v>45688</v>
       </c>
       <c r="B134" t="n">
         <v>0.03074400383563204</v>
       </c>
       <c r="C134" t="n">
-        <v>-0.006027115472455921</v>
+        <v>-0.001813568476578542</v>
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="1" t="n">
+      <c r="A135" s="2" t="n">
         <v>45716</v>
       </c>
       <c r="B135" t="n">
         <v>0.005356171982461908</v>
       </c>
       <c r="C135" t="n">
-        <v>0.005306823159101683</v>
+        <v>0.009634857253662666</v>
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="1" t="n">
+      <c r="A136" s="2" t="n">
         <v>45747</v>
       </c>
       <c r="B136" t="n">
         <v>-0.03936065747103384</v>
       </c>
       <c r="C136" t="n">
-        <v>0.01485239492504366</v>
+        <v>0.01509623143720871</v>
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="1" t="n">
+      <c r="A137" s="2" t="n">
         <v>45777</v>
       </c>
       <c r="B137" t="n">
         <v>-0.0003712512432697251</v>
       </c>
       <c r="C137" t="n">
-        <v>0.04393901351277293</v>
+        <v>0.03992909007029311</v>
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="1" t="n">
+      <c r="A138" s="2" t="n">
         <v>45807</v>
       </c>
       <c r="B138" t="n">
         <v>0.05049871444190139</v>
       </c>
       <c r="C138" t="n">
-        <v>-0.01871251790217808</v>
+        <v>-0.01188025563426093</v>
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="1" t="n">
+      <c r="A139" s="2" t="n">
         <v>45838</v>
       </c>
       <c r="B139" t="n">
         <v>0.043684099601013</v>
       </c>
       <c r="C139" t="n">
-        <v>-0.007032588549490621</v>
+        <v>0.001441935480643254</v>
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="1" t="n">
+      <c r="A140" s="2" t="n">
         <v>45869</v>
       </c>
       <c r="B140" t="n">
         <v>0.01704349688554993</v>
       </c>
       <c r="C140" t="n">
-        <v>-0.003829926806489775</v>
+        <v>-0.005382141263953059</v>
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="1" t="n">
+      <c r="A141" s="2" t="n">
         <v>45898</v>
       </c>
       <c r="B141" t="n">
         <v>0.02376419689285764</v>
       </c>
       <c r="C141" t="n">
-        <v>0.00995042236247335</v>
+        <v>0.01403393362995398</v>
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="1" t="n">
+      <c r="A142" s="2" t="n">
         <v>45930</v>
       </c>
       <c r="B142" t="n">
         <v>0.02752594267972975</v>
       </c>
       <c r="C142" t="n">
-        <v>0.004474673054023581</v>
+        <v>0.0003388793988064812</v>
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="1" t="n">
+      <c r="A143" s="2" t="n">
         <v>45961</v>
       </c>
       <c r="B143" t="n">
         <v>0.02345311271306457</v>
       </c>
       <c r="C143" t="n">
-        <v>-0.015194087086568</v>
+        <v>-0.01025494219471191</v>
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="1" t="n">
+      <c r="A144" s="2" t="n">
         <v>45989</v>
       </c>
       <c r="B144" t="n">
         <v>0.007211569097595304</v>
       </c>
       <c r="C144" t="n">
-        <v>0.0547720052231034</v>
+        <v>0.05066047418057239</v>
       </c>
     </row>
     <row r="145">
-      <c r="A145" s="1" t="n">
+      <c r="A145" s="2" t="n">
         <v>46022</v>
       </c>
       <c r="B145" t="n">
         <v>0.0145794998106231</v>
       </c>
       <c r="C145" t="n">
-        <v>0.003903949545172113</v>
+        <v>0.008206493415200284</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ledoit and Single Factor
</commit_message>
<xml_diff>
--- a/results/monthly_returns.xlsx
+++ b/results/monthly_returns.xlsx
@@ -459,7 +459,7 @@
         <v>-0.03577051251348723</v>
       </c>
       <c r="C2" t="n">
-        <v>-0.00481655169826153</v>
+        <v>-0.0003105142477870728</v>
       </c>
     </row>
     <row r="3">
@@ -470,7 +470,7 @@
         <v>0.05457272646088732</v>
       </c>
       <c r="C3" t="n">
-        <v>0.04729606898759194</v>
+        <v>0.03689612495357093</v>
       </c>
     </row>
     <row r="4">
@@ -481,7 +481,7 @@
         <v>0.007762261335563271</v>
       </c>
       <c r="C4" t="n">
-        <v>0.006338661632828502</v>
+        <v>0.01498246674726625</v>
       </c>
     </row>
     <row r="5">
@@ -492,7 +492,7 @@
         <v>0.01583202208543277</v>
       </c>
       <c r="C5" t="n">
-        <v>0.02011146048383985</v>
+        <v>0.0308741112976096</v>
       </c>
     </row>
     <row r="6">
@@ -503,7 +503,7 @@
         <v>0.01643020929599076</v>
       </c>
       <c r="C6" t="n">
-        <v>0.007680340939861655</v>
+        <v>-0.008809089745784782</v>
       </c>
     </row>
     <row r="7">
@@ -514,7 +514,7 @@
         <v>0.01148059602195001</v>
       </c>
       <c r="C7" t="n">
-        <v>0.006578384151253187</v>
+        <v>0.01932172142390034</v>
       </c>
     </row>
     <row r="8">
@@ -525,7 +525,7 @@
         <v>-0.023164508181366</v>
       </c>
       <c r="C8" t="n">
-        <v>-0.04172244099755235</v>
+        <v>-0.0457627662034269</v>
       </c>
     </row>
     <row r="9">
@@ -536,7 +536,7 @@
         <v>0.02457691833184666</v>
       </c>
       <c r="C9" t="n">
-        <v>0.03003256291393353</v>
+        <v>0.03998821532380905</v>
       </c>
     </row>
     <row r="10">
@@ -547,7 +547,7 @@
         <v>-0.02330935776278098</v>
       </c>
       <c r="C10" t="n">
-        <v>-0.03777058560841617</v>
+        <v>-0.02115908803899224</v>
       </c>
     </row>
     <row r="11">
@@ -558,7 +558,7 @@
         <v>0.004941866289649032</v>
       </c>
       <c r="C11" t="n">
-        <v>0.04772787202912362</v>
+        <v>0.0734984041304949</v>
       </c>
     </row>
     <row r="12">
@@ -569,7 +569,7 @@
         <v>0.02684646801091424</v>
       </c>
       <c r="C12" t="n">
-        <v>0.02867714961939459</v>
+        <v>0.02541264466780386</v>
       </c>
     </row>
     <row r="13">
@@ -580,7 +580,7 @@
         <v>-0.01793837814404243</v>
       </c>
       <c r="C13" t="n">
-        <v>0.005606131058487454</v>
+        <v>0.02526155283915192</v>
       </c>
     </row>
     <row r="14">
@@ -591,7 +591,7 @@
         <v>-0.02282175733578628</v>
       </c>
       <c r="C14" t="n">
-        <v>0.003664408129007701</v>
+        <v>0.01687894808036045</v>
       </c>
     </row>
     <row r="15">
@@ -602,7 +602,7 @@
         <v>0.05685610170123574</v>
       </c>
       <c r="C15" t="n">
-        <v>0.0103595629767555</v>
+        <v>-0.02463691996442547</v>
       </c>
     </row>
     <row r="16">
@@ -613,7 +613,7 @@
         <v>-0.01878225285036577</v>
       </c>
       <c r="C16" t="n">
-        <v>-0.01551358338958826</v>
+        <v>-0.01234506627035867</v>
       </c>
     </row>
     <row r="17">
@@ -624,7 +624,7 @@
         <v>0.02217672013381462</v>
       </c>
       <c r="C17" t="n">
-        <v>0.003728819189570185</v>
+        <v>-0.00897264818147096</v>
       </c>
     </row>
     <row r="18">
@@ -635,7 +635,7 @@
         <v>0.002763819717271396</v>
       </c>
       <c r="C18" t="n">
-        <v>0.01141952297075848</v>
+        <v>0.007552194404542458</v>
       </c>
     </row>
     <row r="19">
@@ -646,7 +646,7 @@
         <v>-0.02380750565336756</v>
       </c>
       <c r="C19" t="n">
-        <v>-0.02379966753639999</v>
+        <v>-0.03392516769170643</v>
       </c>
     </row>
     <row r="20">
@@ -657,7 +657,7 @@
         <v>0.01953878974553074</v>
       </c>
       <c r="C20" t="n">
-        <v>0.04705376305557753</v>
+        <v>0.06493760840647705</v>
       </c>
     </row>
     <row r="21">
@@ -668,7 +668,7 @@
         <v>-0.06371876922900283</v>
       </c>
       <c r="C21" t="n">
-        <v>-0.03222375860079314</v>
+        <v>-0.03509870991545884</v>
       </c>
     </row>
     <row r="22">
@@ -679,7 +679,7 @@
         <v>-0.03029360394779007</v>
       </c>
       <c r="C22" t="n">
-        <v>-0.008770416705412308</v>
+        <v>0.02215385419436208</v>
       </c>
     </row>
     <row r="23">
@@ -690,7 +690,7 @@
         <v>0.07484781831623569</v>
       </c>
       <c r="C23" t="n">
-        <v>0.03254103088179028</v>
+        <v>0.02334413699182387</v>
       </c>
     </row>
     <row r="24">
@@ -701,7 +701,7 @@
         <v>-0.005311215995536839</v>
       </c>
       <c r="C24" t="n">
-        <v>-0.004947861051835726</v>
+        <v>-0.007397723088413953</v>
       </c>
     </row>
     <row r="25">
@@ -712,7 +712,7 @@
         <v>-0.02288379535149846</v>
       </c>
       <c r="C25" t="n">
-        <v>0.021924486432785</v>
+        <v>0.02772523121395692</v>
       </c>
     </row>
     <row r="26">
@@ -723,7 +723,7 @@
         <v>-0.05258465528398181</v>
       </c>
       <c r="C26" t="n">
-        <v>0.007974664155795813</v>
+        <v>0.03486198882517804</v>
       </c>
     </row>
     <row r="27">
@@ -734,7 +734,7 @@
         <v>-0.008168481738206232</v>
       </c>
       <c r="C27" t="n">
-        <v>-0.003837105733913564</v>
+        <v>0.01105539951589406</v>
       </c>
     </row>
     <row r="28">
@@ -745,7 +745,7 @@
         <v>0.07050360052854185</v>
       </c>
       <c r="C28" t="n">
-        <v>0.04918728092849432</v>
+        <v>0.06229177316933843</v>
       </c>
     </row>
     <row r="29">
@@ -756,7 +756,7 @@
         <v>0.01346581614572162</v>
       </c>
       <c r="C29" t="n">
-        <v>0.01755568581401722</v>
+        <v>-0.02294262795329116</v>
       </c>
     </row>
     <row r="30">
@@ -767,7 +767,7 @@
         <v>0.00659258352088357</v>
       </c>
       <c r="C30" t="n">
-        <v>0.01093559364503575</v>
+        <v>0.01516820679664637</v>
       </c>
     </row>
     <row r="31">
@@ -778,7 +778,7 @@
         <v>-0.01362076122737209</v>
       </c>
       <c r="C31" t="n">
-        <v>0.04948549266523025</v>
+        <v>0.08498283108540364</v>
       </c>
     </row>
     <row r="32">
@@ -789,7 +789,7 @@
         <v>0.03674407370358323</v>
       </c>
       <c r="C32" t="n">
-        <v>0.01751486591933996</v>
+        <v>-0.007633916853250226</v>
       </c>
     </row>
     <row r="33">
@@ -800,7 +800,7 @@
         <v>0.002077100500778767</v>
       </c>
       <c r="C33" t="n">
-        <v>-0.04435458387739791</v>
+        <v>-0.0453601444080682</v>
       </c>
     </row>
     <row r="34">
@@ -811,7 +811,7 @@
         <v>0.002306627011404471</v>
       </c>
       <c r="C34" t="n">
-        <v>-0.01263750947580846</v>
+        <v>-0.01615033022771593</v>
       </c>
     </row>
     <row r="35">
@@ -822,7 +822,7 @@
         <v>-0.02102440381119557</v>
       </c>
       <c r="C35" t="n">
-        <v>-0.03559367844640302</v>
+        <v>-0.005899574743832517</v>
       </c>
     </row>
     <row r="36">
@@ -833,7 +833,7 @@
         <v>0.01819181100066963</v>
       </c>
       <c r="C36" t="n">
-        <v>-0.01657266317125299</v>
+        <v>-0.03532277164098992</v>
       </c>
     </row>
     <row r="37">
@@ -844,7 +844,7 @@
         <v>0.03324819018946118</v>
       </c>
       <c r="C37" t="n">
-        <v>0.03049639813702271</v>
+        <v>0.03678202553512994</v>
       </c>
     </row>
     <row r="38">
@@ -855,7 +855,7 @@
         <v>0.01579079678590857</v>
       </c>
       <c r="C38" t="n">
-        <v>0.01269401296900648</v>
+        <v>0.01243933923956877</v>
       </c>
     </row>
     <row r="39">
@@ -866,7 +866,7 @@
         <v>0.02844322118409615</v>
       </c>
       <c r="C39" t="n">
-        <v>0.01727109970099426</v>
+        <v>0.04334061691389333</v>
       </c>
     </row>
     <row r="40">
@@ -877,7 +877,7 @@
         <v>0.01407803634341376</v>
       </c>
       <c r="C40" t="n">
-        <v>0.005368514886413911</v>
+        <v>-0.00294920482624696</v>
       </c>
     </row>
     <row r="41">
@@ -888,7 +888,7 @@
         <v>0.01822042462107884</v>
       </c>
       <c r="C41" t="n">
-        <v>0.03372608753678873</v>
+        <v>0.0092207909058711</v>
       </c>
     </row>
     <row r="42">
@@ -899,7 +899,7 @@
         <v>0.02654951259123661</v>
       </c>
       <c r="C42" t="n">
-        <v>0.02447867586817949</v>
+        <v>0.03092861195275462</v>
       </c>
     </row>
     <row r="43">
@@ -910,7 +910,7 @@
         <v>0.002373678903860118</v>
       </c>
       <c r="C43" t="n">
-        <v>-0.01489892288061603</v>
+        <v>-0.0251574200068704</v>
       </c>
     </row>
     <row r="44">
@@ -921,7 +921,7 @@
         <v>0.02246463779799775</v>
       </c>
       <c r="C44" t="n">
-        <v>0.01620659347711604</v>
+        <v>0.01413086019934311</v>
       </c>
     </row>
     <row r="45">
@@ -932,7 +932,7 @@
         <v>0.00244198517741814</v>
       </c>
       <c r="C45" t="n">
-        <v>-0.04122869241558448</v>
+        <v>0.005638815962982279</v>
       </c>
     </row>
     <row r="46">
@@ -943,7 +943,7 @@
         <v>0.02808540905124245</v>
       </c>
       <c r="C46" t="n">
-        <v>0.006177166231987881</v>
+        <v>-0.01731629803200579</v>
       </c>
     </row>
     <row r="47">
@@ -954,7 +954,7 @@
         <v>0.01894898151901998</v>
       </c>
       <c r="C47" t="n">
-        <v>0.01337724871896624</v>
+        <v>0.03034583913904638</v>
       </c>
     </row>
     <row r="48">
@@ -965,7 +965,7 @@
         <v>0.02194443635302347</v>
       </c>
       <c r="C48" t="n">
-        <v>0.02517856070949299</v>
+        <v>0.04543914642066441</v>
       </c>
     </row>
     <row r="49">
@@ -976,7 +976,7 @@
         <v>0.01303863736857334</v>
       </c>
       <c r="C49" t="n">
-        <v>0.01561468135456912</v>
+        <v>-0.02246681646510476</v>
       </c>
     </row>
     <row r="50">
@@ -987,7 +987,7 @@
         <v>0.04951854951058408</v>
       </c>
       <c r="C50" t="n">
-        <v>-0.01684920269582513</v>
+        <v>-0.03079820814387753</v>
       </c>
     </row>
     <row r="51">
@@ -998,7 +998,7 @@
         <v>-0.04705500135027535</v>
       </c>
       <c r="C51" t="n">
-        <v>-0.06616802133795754</v>
+        <v>-0.06323530838876995</v>
       </c>
     </row>
     <row r="52">
@@ -1009,7 +1009,7 @@
         <v>-0.01795301847933335</v>
       </c>
       <c r="C52" t="n">
-        <v>-0.008152559113326623</v>
+        <v>0.01557257763422526</v>
       </c>
     </row>
     <row r="53">
@@ -1020,7 +1020,7 @@
         <v>0.01261748230660959</v>
       </c>
       <c r="C53" t="n">
-        <v>0.008830318043337011</v>
+        <v>0.009801989374479006</v>
       </c>
     </row>
     <row r="54">
@@ -1031,7 +1031,7 @@
         <v>0.001351174902387803</v>
       </c>
       <c r="C54" t="n">
-        <v>0.01104551890546974</v>
+        <v>-0.02291767995242993</v>
       </c>
     </row>
     <row r="55">
@@ -1042,7 +1042,7 @@
         <v>0.0002616030988843816</v>
       </c>
       <c r="C55" t="n">
-        <v>0.02090510194355684</v>
+        <v>0.03286327766022443</v>
       </c>
     </row>
     <row r="56">
@@ -1053,7 +1053,7 @@
         <v>0.03849477634390881</v>
       </c>
       <c r="C56" t="n">
-        <v>0.01051489736295047</v>
+        <v>0.02993335994857373</v>
       </c>
     </row>
     <row r="57">
@@ -1064,7 +1064,7 @@
         <v>0.008992745924063218</v>
       </c>
       <c r="C57" t="n">
-        <v>0.0208282511001946</v>
+        <v>0.01265583982821303</v>
       </c>
     </row>
     <row r="58">
@@ -1075,7 +1075,7 @@
         <v>0.0066165392530823</v>
       </c>
       <c r="C58" t="n">
-        <v>-0.005263103626727206</v>
+        <v>-0.008040828401230835</v>
       </c>
     </row>
     <row r="59">
@@ -1086,7 +1086,7 @@
         <v>-0.06453623148170358</v>
       </c>
       <c r="C59" t="n">
-        <v>-0.01818643607555086</v>
+        <v>0.01303247056602534</v>
       </c>
     </row>
     <row r="60">
@@ -1097,7 +1097,7 @@
         <v>0.01111789623001095</v>
       </c>
       <c r="C60" t="n">
-        <v>-0.003706219951176296</v>
+        <v>0.02497455449829819</v>
       </c>
     </row>
     <row r="61">
@@ -1108,7 +1108,7 @@
         <v>-0.07816398564554208</v>
       </c>
       <c r="C61" t="n">
-        <v>-0.06307783494331633</v>
+        <v>-0.04772245244698381</v>
       </c>
     </row>
     <row r="62">
@@ -1119,7 +1119,7 @@
         <v>0.07601880736345278</v>
       </c>
       <c r="C62" t="n">
-        <v>0.02063107719080389</v>
+        <v>0.02631517040947831</v>
       </c>
     </row>
     <row r="63">
@@ -1130,7 +1130,7 @@
         <v>0.03326236662472595</v>
       </c>
       <c r="C63" t="n">
-        <v>0.03825593402676782</v>
+        <v>0.0452605980970987</v>
       </c>
     </row>
     <row r="64">
@@ -1141,7 +1141,7 @@
         <v>0.01472293864230933</v>
       </c>
       <c r="C64" t="n">
-        <v>0.03494084912618512</v>
+        <v>0.03790064509125353</v>
       </c>
     </row>
     <row r="65">
@@ -1152,7 +1152,7 @@
         <v>0.03766175186714266</v>
       </c>
       <c r="C65" t="n">
-        <v>0.02737376576035037</v>
+        <v>0.0146451918659667</v>
       </c>
     </row>
     <row r="66">
@@ -1163,7 +1163,7 @@
         <v>-0.06023474533191252</v>
       </c>
       <c r="C66" t="n">
-        <v>-0.02222157984850629</v>
+        <v>-0.003630259120516551</v>
       </c>
     </row>
     <row r="67">
@@ -1174,7 +1174,7 @@
         <v>0.07033903461068169</v>
       </c>
       <c r="C67" t="n">
-        <v>0.04186613772142073</v>
+        <v>0.03723087912617451</v>
       </c>
     </row>
     <row r="68">
@@ -1185,7 +1185,7 @@
         <v>0.00439947754685985</v>
       </c>
       <c r="C68" t="n">
-        <v>0.009522815551679513</v>
+        <v>0.00600799830687519</v>
       </c>
     </row>
     <row r="69">
@@ -1196,7 +1196,7 @@
         <v>-0.01828779657461423</v>
       </c>
       <c r="C69" t="n">
-        <v>0.0152103331585349</v>
+        <v>0.04770704412031702</v>
       </c>
     </row>
     <row r="70">
@@ -1207,7 +1207,7 @@
         <v>0.02466315429160364</v>
       </c>
       <c r="C70" t="n">
-        <v>0.006604812653261417</v>
+        <v>0.02075205425050233</v>
       </c>
     </row>
     <row r="71">
@@ -1218,7 +1218,7 @@
         <v>0.02217750538357088</v>
       </c>
       <c r="C71" t="n">
-        <v>-0.001327221783458397</v>
+        <v>-0.01353477375880567</v>
       </c>
     </row>
     <row r="72">
@@ -1229,7 +1229,7 @@
         <v>0.02997799889267743</v>
       </c>
       <c r="C72" t="n">
-        <v>0.01873125958053234</v>
+        <v>-0.01085737135356558</v>
       </c>
     </row>
     <row r="73">
@@ -1240,7 +1240,7 @@
         <v>0.03482421028928007</v>
       </c>
       <c r="C73" t="n">
-        <v>0.04193944098221207</v>
+        <v>0.03293717581675445</v>
       </c>
     </row>
     <row r="74">
@@ -1251,7 +1251,7 @@
         <v>-0.009580265949088524</v>
       </c>
       <c r="C74" t="n">
-        <v>0.01169955204495742</v>
+        <v>0.05566482369506633</v>
       </c>
     </row>
     <row r="75">
@@ -1262,7 +1262,7 @@
         <v>-0.08791498768503248</v>
       </c>
       <c r="C75" t="n">
-        <v>-0.08547222154564432</v>
+        <v>-0.09382759038766579</v>
       </c>
     </row>
     <row r="76">
@@ -1273,7 +1273,7 @@
         <v>-0.1306650921429244</v>
       </c>
       <c r="C76" t="n">
-        <v>-0.1177459164809954</v>
+        <v>-0.070551743397304</v>
       </c>
     </row>
     <row r="77">
@@ -1284,7 +1284,7 @@
         <v>0.1075112783889687</v>
       </c>
       <c r="C77" t="n">
-        <v>0.107370588150448</v>
+        <v>0.04667309877695485</v>
       </c>
     </row>
     <row r="78">
@@ -1295,7 +1295,7 @@
         <v>0.04142078875265022</v>
       </c>
       <c r="C78" t="n">
-        <v>0.0261562079345386</v>
+        <v>0.03454819857257937</v>
       </c>
     </row>
     <row r="79">
@@ -1306,7 +1306,7 @@
         <v>0.02854315181783309</v>
       </c>
       <c r="C79" t="n">
-        <v>-0.01060515899879751</v>
+        <v>-0.02892670705260554</v>
       </c>
     </row>
     <row r="80">
@@ -1317,7 +1317,7 @@
         <v>0.04883592322798035</v>
       </c>
       <c r="C80" t="n">
-        <v>0.07148084680712641</v>
+        <v>0.07548018795773868</v>
       </c>
     </row>
     <row r="81">
@@ -1328,7 +1328,7 @@
         <v>0.06540930795489953</v>
       </c>
       <c r="C81" t="n">
-        <v>0.03204056865028183</v>
+        <v>-0.01859328917869386</v>
       </c>
     </row>
     <row r="82">
@@ -1339,7 +1339,7 @@
         <v>-0.03798082063905267</v>
       </c>
       <c r="C82" t="n">
-        <v>-0.01792825628676786</v>
+        <v>0.0001998800906176534</v>
       </c>
     </row>
     <row r="83">
@@ -1350,7 +1350,7 @@
         <v>-0.03589474696672947</v>
       </c>
       <c r="C83" t="n">
-        <v>-0.01878108115765808</v>
+        <v>0.01045654691778345</v>
       </c>
     </row>
     <row r="84">
@@ -1361,7 +1361,7 @@
         <v>0.1283940181539289</v>
       </c>
       <c r="C84" t="n">
-        <v>0.07259584873826545</v>
+        <v>0.01387373353078162</v>
       </c>
     </row>
     <row r="85">
@@ -1372,7 +1372,7 @@
         <v>0.03983956548531003</v>
       </c>
       <c r="C85" t="n">
-        <v>0.0289022890468589</v>
+        <v>-0.001394935734889661</v>
       </c>
     </row>
     <row r="86">
@@ -1383,7 +1383,7 @@
         <v>-0.01212400733186289</v>
       </c>
       <c r="C86" t="n">
-        <v>-0.005245280012396868</v>
+        <v>-0.01965965077570352</v>
       </c>
     </row>
     <row r="87">
@@ -1394,7 +1394,7 @@
         <v>0.02733062300679211</v>
       </c>
       <c r="C87" t="n">
-        <v>-0.004572640806403129</v>
+        <v>-0.04341570182356316</v>
       </c>
     </row>
     <row r="88">
@@ -1405,7 +1405,7 @@
         <v>0.04536283607748608</v>
       </c>
       <c r="C88" t="n">
-        <v>0.08262019648589847</v>
+        <v>0.111363065630386</v>
       </c>
     </row>
     <row r="89">
@@ -1416,7 +1416,7 @@
         <v>0.05016847426313767</v>
       </c>
       <c r="C89" t="n">
-        <v>0.02432179160466919</v>
+        <v>0.03414583541110992</v>
       </c>
     </row>
     <row r="90">
@@ -1427,7 +1427,7 @@
         <v>0.02015621412882964</v>
       </c>
       <c r="C90" t="n">
-        <v>0.02393516928225115</v>
+        <v>-0.00330748347211761</v>
       </c>
     </row>
     <row r="91">
@@ -1438,7 +1438,7 @@
         <v>0.009085467039068967</v>
       </c>
       <c r="C91" t="n">
-        <v>-0.01672115604024303</v>
+        <v>-0.01782574837363823</v>
       </c>
     </row>
     <row r="92">
@@ -1449,7 +1449,7 @@
         <v>0.01882876021698834</v>
       </c>
       <c r="C92" t="n">
-        <v>0.02842117726803394</v>
+        <v>0.03792584062635949</v>
       </c>
     </row>
     <row r="93">
@@ -1460,7 +1460,7 @@
         <v>0.02292599245632672</v>
       </c>
       <c r="C93" t="n">
-        <v>0.007994830845347073</v>
+        <v>0.01685489366687223</v>
       </c>
     </row>
     <row r="94">
@@ -1471,7 +1471,7 @@
         <v>-0.04484438196599666</v>
       </c>
       <c r="C94" t="n">
-        <v>-0.05847634547353054</v>
+        <v>-0.06144338363020276</v>
       </c>
     </row>
     <row r="95">
@@ -1482,7 +1482,7 @@
         <v>0.06369195815598885</v>
       </c>
       <c r="C95" t="n">
-        <v>0.03517308509824792</v>
+        <v>0.03498712401650843</v>
       </c>
     </row>
     <row r="96">
@@ -1493,7 +1493,7 @@
         <v>-0.01485364644369896</v>
       </c>
       <c r="C96" t="n">
-        <v>-0.03091858192901106</v>
+        <v>-0.01284309109342264</v>
       </c>
     </row>
     <row r="97">
@@ -1504,7 +1504,7 @@
         <v>0.05275242494481132</v>
       </c>
       <c r="C97" t="n">
-        <v>0.08029981468635675</v>
+        <v>0.1042569325032066</v>
       </c>
     </row>
     <row r="98">
@@ -1515,7 +1515,7 @@
         <v>-0.04101565747775374</v>
       </c>
       <c r="C98" t="n">
-        <v>-0.01778649764724247</v>
+        <v>-0.01872646799851295</v>
       </c>
     </row>
     <row r="99">
@@ -1526,7 +1526,7 @@
         <v>-0.02440661653703706</v>
       </c>
       <c r="C99" t="n">
-        <v>-0.01232212651185563</v>
+        <v>-0.02193601230567215</v>
       </c>
     </row>
     <row r="100">
@@ -1537,7 +1537,7 @@
         <v>0.02739841992527333</v>
       </c>
       <c r="C100" t="n">
-        <v>0.04908304111674888</v>
+        <v>0.07335561073606392</v>
       </c>
     </row>
     <row r="101">
@@ -1548,7 +1548,7 @@
         <v>-0.07246087523648355</v>
       </c>
       <c r="C101" t="n">
-        <v>-0.03172862178691287</v>
+        <v>-0.0179008385124533</v>
       </c>
     </row>
     <row r="102">
@@ -1559,7 +1559,7 @@
         <v>0.005871650263511217</v>
       </c>
       <c r="C102" t="n">
-        <v>0.01051186310250954</v>
+        <v>0.02009885418086607</v>
       </c>
     </row>
     <row r="103">
@@ -1570,7 +1570,7 @@
         <v>-0.08596805176643892</v>
       </c>
       <c r="C103" t="n">
-        <v>-0.05507990205327662</v>
+        <v>-0.04406468390315271</v>
       </c>
     </row>
     <row r="104">
@@ -1581,7 +1581,7 @@
         <v>0.07919681433848735</v>
       </c>
       <c r="C104" t="n">
-        <v>0.03604613722076366</v>
+        <v>0.03671534962841447</v>
       </c>
     </row>
     <row r="105">
@@ -1592,7 +1592,7 @@
         <v>-0.04332771130830771</v>
       </c>
       <c r="C105" t="n">
-        <v>-0.02626497467782272</v>
+        <v>-0.01206392080510591</v>
       </c>
     </row>
     <row r="106">
@@ -1603,7 +1603,7 @@
         <v>-0.09169976227284632</v>
       </c>
       <c r="C106" t="n">
-        <v>-0.08290421413523899</v>
+        <v>-0.10868744661239</v>
       </c>
     </row>
     <row r="107">
@@ -1614,7 +1614,7 @@
         <v>0.08600326884212639</v>
       </c>
       <c r="C107" t="n">
-        <v>0.06998622899605189</v>
+        <v>0.04089771109805466</v>
       </c>
     </row>
     <row r="108">
@@ -1625,7 +1625,7 @@
         <v>0.07019817439074505</v>
       </c>
       <c r="C108" t="n">
-        <v>0.05977169149329654</v>
+        <v>0.06602485881457602</v>
       </c>
     </row>
     <row r="109">
@@ -1636,7 +1636,7 @@
         <v>-0.04196388752670809</v>
       </c>
       <c r="C109" t="n">
-        <v>-0.02823064212783596</v>
+        <v>-0.01318339147667644</v>
       </c>
     </row>
     <row r="110">
@@ -1647,7 +1647,7 @@
         <v>0.06616089743523371</v>
       </c>
       <c r="C110" t="n">
-        <v>0.02393514447393397</v>
+        <v>0.002875139997772318</v>
       </c>
     </row>
     <row r="111">
@@ -1658,7 +1658,7 @@
         <v>-0.02239431803222399</v>
       </c>
       <c r="C111" t="n">
-        <v>-0.006891280812889752</v>
+        <v>-0.02474469546834168</v>
       </c>
     </row>
     <row r="112">
@@ -1669,7 +1669,7 @@
         <v>0.03122580989791321</v>
       </c>
       <c r="C112" t="n">
-        <v>0.0118421415057038</v>
+        <v>0.04239179308824732</v>
       </c>
     </row>
     <row r="113">
@@ -1680,7 +1680,7 @@
         <v>0.02644255003476621</v>
       </c>
       <c r="C113" t="n">
-        <v>0.02734082497437937</v>
+        <v>0.02705486454363022</v>
       </c>
     </row>
     <row r="114">
@@ -1691,7 +1691,7 @@
         <v>-0.01825027086054789</v>
       </c>
       <c r="C114" t="n">
-        <v>-0.04681455207830134</v>
+        <v>-0.04845953275123581</v>
       </c>
     </row>
     <row r="115">
@@ -1702,7 +1702,7 @@
         <v>0.06093188600225954</v>
       </c>
       <c r="C115" t="n">
-        <v>0.01631181051322894</v>
+        <v>0.01500055557102448</v>
       </c>
     </row>
     <row r="116">
@@ -1713,7 +1713,7 @@
         <v>0.0290835962367811</v>
       </c>
       <c r="C116" t="n">
-        <v>0.008283814823725661</v>
+        <v>0.0005305220785111506</v>
       </c>
     </row>
     <row r="117">
@@ -1724,7 +1724,7 @@
         <v>-0.02253641802697804</v>
       </c>
       <c r="C117" t="n">
-        <v>-0.02450943501530416</v>
+        <v>-0.03776670294666797</v>
       </c>
     </row>
     <row r="118">
@@ -1735,7 +1735,7 @@
         <v>-0.04645542708300802</v>
       </c>
       <c r="C118" t="n">
-        <v>-0.04398133864991243</v>
+        <v>-0.04777652959331547</v>
       </c>
     </row>
     <row r="119">
@@ -1746,7 +1746,7 @@
         <v>-0.02171054624420314</v>
       </c>
       <c r="C119" t="n">
-        <v>-0.01101723542670296</v>
+        <v>-0.01508717164337134</v>
       </c>
     </row>
     <row r="120">
@@ -1757,7 +1757,7 @@
         <v>0.09051414707262974</v>
       </c>
       <c r="C120" t="n">
-        <v>0.03459969159971101</v>
+        <v>0.0432068723932937</v>
       </c>
     </row>
     <row r="121">
@@ -1768,7 +1768,7 @@
         <v>0.04513240680873794</v>
       </c>
       <c r="C121" t="n">
-        <v>0.01908374117738183</v>
+        <v>0.02827663873638394</v>
       </c>
     </row>
     <row r="122">
@@ -1779,7 +1779,7 @@
         <v>0.01245418746238778</v>
       </c>
       <c r="C122" t="n">
-        <v>-0.002972561984548144</v>
+        <v>-9.057499107558049e-06</v>
       </c>
     </row>
     <row r="123">
@@ -1790,7 +1790,7 @@
         <v>0.03901825082531514</v>
       </c>
       <c r="C123" t="n">
-        <v>0.02182263764553104</v>
+        <v>0.009578315880778603</v>
       </c>
     </row>
     <row r="124">
@@ -1801,7 +1801,7 @@
         <v>0.03637442820614256</v>
       </c>
       <c r="C124" t="n">
-        <v>0.02766588670083584</v>
+        <v>0.03817348813934573</v>
       </c>
     </row>
     <row r="125">
@@ -1812,7 +1812,7 @@
         <v>-0.03609511822437324</v>
       </c>
       <c r="C125" t="n">
-        <v>0.007887485409802872</v>
+        <v>-9.293926549834488e-05</v>
       </c>
     </row>
     <row r="126">
@@ -1823,7 +1823,7 @@
         <v>0.05159895294222033</v>
       </c>
       <c r="C126" t="n">
-        <v>0.03008781794761481</v>
+        <v>0.01877852763371078</v>
       </c>
     </row>
     <row r="127">
@@ -1834,7 +1834,7 @@
         <v>0.01673400189527829</v>
       </c>
       <c r="C127" t="n">
-        <v>-0.01003117137510173</v>
+        <v>-0.01772801294387442</v>
       </c>
     </row>
     <row r="128">
@@ -1845,7 +1845,7 @@
         <v>0.01638886236175519</v>
       </c>
       <c r="C128" t="n">
-        <v>0.0273998663907862</v>
+        <v>0.04988939134366609</v>
       </c>
     </row>
     <row r="129">
@@ -1856,7 +1856,7 @@
         <v>0.02662711852757172</v>
       </c>
       <c r="C129" t="n">
-        <v>0.04480272094453801</v>
+        <v>0.06297685061879238</v>
       </c>
     </row>
     <row r="130">
@@ -1867,7 +1867,7 @@
         <v>0.01491367792089069</v>
       </c>
       <c r="C130" t="n">
-        <v>-0.005980811556354734</v>
+        <v>0.01565535143889565</v>
       </c>
     </row>
     <row r="131">
@@ -1878,7 +1878,7 @@
         <v>-0.02230215658726872</v>
       </c>
       <c r="C131" t="n">
-        <v>-0.04647168819412067</v>
+        <v>-0.0379558456167232</v>
       </c>
     </row>
     <row r="132">
@@ -1889,7 +1889,7 @@
         <v>0.04154212052715963</v>
       </c>
       <c r="C132" t="n">
-        <v>-6.588281982651892e-05</v>
+        <v>0.02828676061233982</v>
       </c>
     </row>
     <row r="133">
@@ -1900,7 +1900,7 @@
         <v>-0.03216767101109499</v>
       </c>
       <c r="C133" t="n">
-        <v>-0.03434676809823738</v>
+        <v>-0.0540783593306607</v>
       </c>
     </row>
     <row r="134">
@@ -1911,7 +1911,7 @@
         <v>0.03074400383563204</v>
       </c>
       <c r="C134" t="n">
-        <v>-0.001813568476578542</v>
+        <v>0.004570192219349434</v>
       </c>
     </row>
     <row r="135">
@@ -1922,7 +1922,7 @@
         <v>0.005356171982461908</v>
       </c>
       <c r="C135" t="n">
-        <v>0.009634857253662666</v>
+        <v>0.04017696490145747</v>
       </c>
     </row>
     <row r="136">
@@ -1933,7 +1933,7 @@
         <v>-0.03936065747103384</v>
       </c>
       <c r="C136" t="n">
-        <v>0.01509623143720871</v>
+        <v>0.01567881282290447</v>
       </c>
     </row>
     <row r="137">
@@ -1944,7 +1944,7 @@
         <v>-0.0003712512432697251</v>
       </c>
       <c r="C137" t="n">
-        <v>0.03992909007029311</v>
+        <v>0.01874150659207298</v>
       </c>
     </row>
     <row r="138">
@@ -1955,7 +1955,7 @@
         <v>0.05049871444190139</v>
       </c>
       <c r="C138" t="n">
-        <v>-0.01188025563426093</v>
+        <v>-0.02178318237543584</v>
       </c>
     </row>
     <row r="139">
@@ -1966,7 +1966,7 @@
         <v>0.043684099601013</v>
       </c>
       <c r="C139" t="n">
-        <v>0.001441935480643254</v>
+        <v>-0.01643574938163797</v>
       </c>
     </row>
     <row r="140">
@@ -1977,7 +1977,7 @@
         <v>0.01704349688554993</v>
       </c>
       <c r="C140" t="n">
-        <v>-0.005382141263953059</v>
+        <v>0.009004327073858814</v>
       </c>
     </row>
     <row r="141">
@@ -1988,7 +1988,7 @@
         <v>0.02376419689285764</v>
       </c>
       <c r="C141" t="n">
-        <v>0.01403393362995398</v>
+        <v>-0.001328872723476929</v>
       </c>
     </row>
     <row r="142">
@@ -1999,7 +1999,7 @@
         <v>0.02752594267972975</v>
       </c>
       <c r="C142" t="n">
-        <v>0.0003388793988064812</v>
+        <v>0.01100461834777438</v>
       </c>
     </row>
     <row r="143">
@@ -2010,7 +2010,7 @@
         <v>0.02345311271306457</v>
       </c>
       <c r="C143" t="n">
-        <v>-0.01025494219471191</v>
+        <v>-0.01937788211653691</v>
       </c>
     </row>
     <row r="144">
@@ -2021,7 +2021,7 @@
         <v>0.007211569097595304</v>
       </c>
       <c r="C144" t="n">
-        <v>0.05066047418057239</v>
+        <v>0.04493337226460223</v>
       </c>
     </row>
     <row r="145">
@@ -2032,7 +2032,7 @@
         <v>0.0145794998106231</v>
       </c>
       <c r="C145" t="n">
-        <v>0.008206493415200284</v>
+        <v>-0.0180947024901323</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update final notebook and results
</commit_message>
<xml_diff>
--- a/results/monthly_returns.xlsx
+++ b/results/monthly_returns.xlsx
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,24 +45,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -435,101 +421,101 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>VW</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>MVP</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="1" t="n">
         <v>41670</v>
       </c>
       <c r="B2" t="n">
         <v>-0.03466947681484572</v>
       </c>
       <c r="C2" t="n">
-        <v>-0.004816551698261532</v>
+        <v>-0.004816551698261525</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="1" t="n">
         <v>41698</v>
       </c>
       <c r="B3" t="n">
         <v>0.05448901058685536</v>
       </c>
       <c r="C3" t="n">
-        <v>0.04729606898759196</v>
+        <v>0.04729606898759198</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="1" t="n">
         <v>41729</v>
       </c>
       <c r="B4" t="n">
         <v>0.005675374213538538</v>
       </c>
       <c r="C4" t="n">
-        <v>0.006338661632828495</v>
+        <v>0.006338661632828478</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="1" t="n">
         <v>41759</v>
       </c>
       <c r="B5" t="n">
         <v>0.01488919032874131</v>
       </c>
       <c r="C5" t="n">
-        <v>0.02011146048383987</v>
+        <v>0.02011146048383988</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="1" t="n">
         <v>41789</v>
       </c>
       <c r="B6" t="n">
         <v>0.01636391439529787</v>
       </c>
       <c r="C6" t="n">
-        <v>0.00768034093986167</v>
+        <v>0.007680340939861668</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="1" t="n">
         <v>41820</v>
       </c>
       <c r="B7" t="n">
         <v>0.01156724461757659</v>
       </c>
       <c r="C7" t="n">
-        <v>0.006578384151253175</v>
+        <v>0.006578384151253172</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="1" t="n">
         <v>41851</v>
       </c>
       <c r="B8" t="n">
         <v>-0.0231891554867019</v>
       </c>
       <c r="C8" t="n">
-        <v>-0.04172244099755237</v>
+        <v>-0.04172244099755239</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="1" t="n">
         <v>41880</v>
       </c>
       <c r="B9" t="n">
@@ -540,29 +526,29 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="1" t="n">
         <v>41912</v>
       </c>
       <c r="B10" t="n">
         <v>-0.02382859395994193</v>
       </c>
       <c r="C10" t="n">
-        <v>-0.03777058560841619</v>
+        <v>-0.0377705856084162</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="1" t="n">
         <v>41943</v>
       </c>
       <c r="B11" t="n">
         <v>0.004460323367332387</v>
       </c>
       <c r="C11" t="n">
-        <v>0.04772787202912362</v>
+        <v>0.04772787202912363</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="1" t="n">
         <v>41971</v>
       </c>
       <c r="B12" t="n">
@@ -573,73 +559,73 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="1" t="n">
         <v>42004</v>
       </c>
       <c r="B13" t="n">
         <v>-0.01799112371716742</v>
       </c>
       <c r="C13" t="n">
-        <v>0.005606131058487443</v>
+        <v>0.005606131058487441</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="1" t="n">
         <v>42034</v>
       </c>
       <c r="B14" t="n">
         <v>-0.02342449533152584</v>
       </c>
       <c r="C14" t="n">
-        <v>0.00357075004108983</v>
+        <v>0.003570750041089836</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n">
+      <c r="A15" s="1" t="n">
         <v>42062</v>
       </c>
       <c r="B15" t="n">
         <v>0.05743351221882392</v>
       </c>
       <c r="C15" t="n">
-        <v>0.01038524096918348</v>
+        <v>0.01038524096918349</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
+      <c r="A16" s="1" t="n">
         <v>42094</v>
       </c>
       <c r="B16" t="n">
         <v>-0.01939266312056785</v>
       </c>
       <c r="C16" t="n">
-        <v>-0.01552099784555949</v>
+        <v>-0.01552099784555951</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n">
+      <c r="A17" s="1" t="n">
         <v>42124</v>
       </c>
       <c r="B17" t="n">
         <v>0.02259155532991046</v>
       </c>
       <c r="C17" t="n">
-        <v>0.003733928655914372</v>
+        <v>0.003733928655914378</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n">
+      <c r="A18" s="1" t="n">
         <v>42153</v>
       </c>
       <c r="B18" t="n">
         <v>0.002463010060876067</v>
       </c>
       <c r="C18" t="n">
-        <v>0.01146074004867236</v>
+        <v>0.01146074004867237</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n">
+      <c r="A19" s="1" t="n">
         <v>42185</v>
       </c>
       <c r="B19" t="n">
@@ -650,40 +636,40 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
+      <c r="A20" s="1" t="n">
         <v>42216</v>
       </c>
       <c r="B20" t="n">
         <v>0.01974227665896659</v>
       </c>
       <c r="C20" t="n">
-        <v>0.04706859901513759</v>
+        <v>0.04706859901513761</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n">
+      <c r="A21" s="1" t="n">
         <v>42247</v>
       </c>
       <c r="B21" t="n">
         <v>-0.06383686467522161</v>
       </c>
       <c r="C21" t="n">
-        <v>-0.03215867052727071</v>
+        <v>-0.03215867052727073</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n">
+      <c r="A22" s="1" t="n">
         <v>42277</v>
       </c>
       <c r="B22" t="n">
         <v>-0.03083580228045991</v>
       </c>
       <c r="C22" t="n">
-        <v>-0.008706334732225998</v>
+        <v>-0.008706334732226002</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n">
+      <c r="A23" s="1" t="n">
         <v>42307</v>
       </c>
       <c r="B23" t="n">
@@ -694,51 +680,51 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n">
+      <c r="A24" s="1" t="n">
         <v>42338</v>
       </c>
       <c r="B24" t="n">
         <v>-0.005802098631818281</v>
       </c>
       <c r="C24" t="n">
-        <v>-0.00500362658464126</v>
+        <v>-0.005003626584641258</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n">
+      <c r="A25" s="1" t="n">
         <v>42369</v>
       </c>
       <c r="B25" t="n">
         <v>-0.02284281854976636</v>
       </c>
       <c r="C25" t="n">
-        <v>0.02188974998914273</v>
+        <v>0.02188974998914272</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n">
+      <c r="A26" s="1" t="n">
         <v>42398</v>
       </c>
       <c r="B26" t="n">
         <v>-0.05314231765160421</v>
       </c>
       <c r="C26" t="n">
-        <v>0.008037784551388497</v>
+        <v>0.00803778455138849</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="n">
+      <c r="A27" s="1" t="n">
         <v>42429</v>
       </c>
       <c r="B27" t="n">
         <v>-0.008092464026211086</v>
       </c>
       <c r="C27" t="n">
-        <v>-0.003840527991693734</v>
+        <v>-0.003840527991693743</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n">
+      <c r="A28" s="1" t="n">
         <v>42460</v>
       </c>
       <c r="B28" t="n">
@@ -749,7 +735,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n">
+      <c r="A29" s="1" t="n">
         <v>42489</v>
       </c>
       <c r="B29" t="n">
@@ -760,29 +746,29 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n">
+      <c r="A30" s="1" t="n">
         <v>42521</v>
       </c>
       <c r="B30" t="n">
         <v>0.006548422811811738</v>
       </c>
       <c r="C30" t="n">
-        <v>0.01093742601190668</v>
+        <v>0.0109374260119067</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n">
+      <c r="A31" s="1" t="n">
         <v>42551</v>
       </c>
       <c r="B31" t="n">
         <v>-0.01460192200764904</v>
       </c>
       <c r="C31" t="n">
-        <v>0.04961961275709112</v>
+        <v>0.04961961275709108</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n">
+      <c r="A32" s="1" t="n">
         <v>42580</v>
       </c>
       <c r="B32" t="n">
@@ -793,7 +779,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n">
+      <c r="A33" s="1" t="n">
         <v>42613</v>
       </c>
       <c r="B33" t="n">
@@ -804,7 +790,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n">
+      <c r="A34" s="1" t="n">
         <v>42643</v>
       </c>
       <c r="B34" t="n">
@@ -815,73 +801,73 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="n">
+      <c r="A35" s="1" t="n">
         <v>42674</v>
       </c>
       <c r="B35" t="n">
         <v>-0.02058439880700975</v>
       </c>
       <c r="C35" t="n">
-        <v>-0.03576779358297394</v>
+        <v>-0.03576779358297397</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n">
+      <c r="A36" s="1" t="n">
         <v>42704</v>
       </c>
       <c r="B36" t="n">
         <v>0.01816491203159422</v>
       </c>
       <c r="C36" t="n">
-        <v>-0.01658175311627109</v>
+        <v>-0.01658175311627108</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n">
+      <c r="A37" s="1" t="n">
         <v>42734</v>
       </c>
       <c r="B37" t="n">
         <v>0.03306895540304732</v>
       </c>
       <c r="C37" t="n">
-        <v>0.03049911660827729</v>
+        <v>0.03049911660827727</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n">
+      <c r="A38" s="1" t="n">
         <v>42766</v>
       </c>
       <c r="B38" t="n">
         <v>0.0158552326211697</v>
       </c>
       <c r="C38" t="n">
-        <v>0.01269401296900649</v>
+        <v>0.0126940129690065</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="n">
+      <c r="A39" s="1" t="n">
         <v>42794</v>
       </c>
       <c r="B39" t="n">
         <v>0.02841716053931977</v>
       </c>
       <c r="C39" t="n">
-        <v>0.01727109970099421</v>
+        <v>0.01727109970099422</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n">
+      <c r="A40" s="1" t="n">
         <v>42825</v>
       </c>
       <c r="B40" t="n">
         <v>0.01381472660672422</v>
       </c>
       <c r="C40" t="n">
-        <v>0.005368514886413949</v>
+        <v>0.005368514886413947</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="n">
+      <c r="A41" s="1" t="n">
         <v>42853</v>
       </c>
       <c r="B41" t="n">
@@ -892,40 +878,40 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n">
+      <c r="A42" s="1" t="n">
         <v>42886</v>
       </c>
       <c r="B42" t="n">
         <v>0.02651773788834572</v>
       </c>
       <c r="C42" t="n">
-        <v>0.0244786758681795</v>
+        <v>0.02447867586817952</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="n">
+      <c r="A43" s="1" t="n">
         <v>42916</v>
       </c>
       <c r="B43" t="n">
         <v>0.002591194011971239</v>
       </c>
       <c r="C43" t="n">
-        <v>-0.01489892288061605</v>
+        <v>-0.01489892288061604</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n">
+      <c r="A44" s="1" t="n">
         <v>42947</v>
       </c>
       <c r="B44" t="n">
         <v>0.02243783635412428</v>
       </c>
       <c r="C44" t="n">
-        <v>0.01620659347711608</v>
+        <v>0.01620659347711607</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n">
+      <c r="A45" s="1" t="n">
         <v>42978</v>
       </c>
       <c r="B45" t="n">
@@ -936,18 +922,18 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n">
+      <c r="A46" s="1" t="n">
         <v>43007</v>
       </c>
       <c r="B46" t="n">
         <v>0.02826316604636436</v>
       </c>
       <c r="C46" t="n">
-        <v>0.006177166231987849</v>
+        <v>0.006177166231987861</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="n">
+      <c r="A47" s="1" t="n">
         <v>43039</v>
       </c>
       <c r="B47" t="n">
@@ -958,62 +944,62 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="n">
+      <c r="A48" s="1" t="n">
         <v>43069</v>
       </c>
       <c r="B48" t="n">
         <v>0.02189215041849694</v>
       </c>
       <c r="C48" t="n">
-        <v>0.02517856070949296</v>
+        <v>0.02517856070949299</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="n">
+      <c r="A49" s="1" t="n">
         <v>43098</v>
       </c>
       <c r="B49" t="n">
         <v>0.01298604820737139</v>
       </c>
       <c r="C49" t="n">
-        <v>0.01561468135456914</v>
+        <v>0.01561468135456915</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="n">
+      <c r="A50" s="1" t="n">
         <v>43131</v>
       </c>
       <c r="B50" t="n">
         <v>0.0495426516953796</v>
       </c>
       <c r="C50" t="n">
-        <v>-0.01684841794160993</v>
+        <v>-0.01684841794160994</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="n">
+      <c r="A51" s="1" t="n">
         <v>43159</v>
       </c>
       <c r="B51" t="n">
         <v>-0.04703929558467417</v>
       </c>
       <c r="C51" t="n">
-        <v>-0.06616790740477092</v>
+        <v>-0.06616790740477094</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="n">
+      <c r="A52" s="1" t="n">
         <v>43189</v>
       </c>
       <c r="B52" t="n">
         <v>-0.01795800966767334</v>
       </c>
       <c r="C52" t="n">
-        <v>-0.008152965052309042</v>
+        <v>-0.008152965052309039</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="n">
+      <c r="A53" s="1" t="n">
         <v>43220</v>
       </c>
       <c r="B53" t="n">
@@ -1024,18 +1010,18 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="n">
+      <c r="A54" s="1" t="n">
         <v>43251</v>
       </c>
       <c r="B54" t="n">
         <v>0.001630562844733072</v>
       </c>
       <c r="C54" t="n">
-        <v>0.01104570981046299</v>
+        <v>0.01104570981046301</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="n">
+      <c r="A55" s="1" t="n">
         <v>43280</v>
       </c>
       <c r="B55" t="n">
@@ -1046,7 +1032,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="n">
+      <c r="A56" s="1" t="n">
         <v>43312</v>
       </c>
       <c r="B56" t="n">
@@ -1057,7 +1043,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="n">
+      <c r="A57" s="1" t="n">
         <v>43343</v>
       </c>
       <c r="B57" t="n">
@@ -1068,18 +1054,18 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="n">
+      <c r="A58" s="1" t="n">
         <v>43371</v>
       </c>
       <c r="B58" t="n">
         <v>0.0065039867209985</v>
       </c>
       <c r="C58" t="n">
-        <v>-0.00526320174439034</v>
+        <v>-0.005263201744390336</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="n">
+      <c r="A59" s="1" t="n">
         <v>43404</v>
       </c>
       <c r="B59" t="n">
@@ -1090,183 +1076,183 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="n">
+      <c r="A60" s="1" t="n">
         <v>43434</v>
       </c>
       <c r="B60" t="n">
         <v>0.01104817414805632</v>
       </c>
       <c r="C60" t="n">
-        <v>-0.003706218250993612</v>
+        <v>-0.003706218250993618</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="n">
+      <c r="A61" s="1" t="n">
         <v>43465</v>
       </c>
       <c r="B61" t="n">
         <v>-0.07818106311506255</v>
       </c>
       <c r="C61" t="n">
-        <v>-0.063077935376483</v>
+        <v>-0.06307793537648301</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="n">
+      <c r="A62" s="1" t="n">
         <v>43496</v>
       </c>
       <c r="B62" t="n">
         <v>0.0763907547289818</v>
       </c>
       <c r="C62" t="n">
-        <v>0.02063107719080389</v>
+        <v>0.0206310771908039</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="n">
+      <c r="A63" s="1" t="n">
         <v>43524</v>
       </c>
       <c r="B63" t="n">
         <v>0.03324696658975932</v>
       </c>
       <c r="C63" t="n">
-        <v>0.03825593402676784</v>
+        <v>0.03825593402676786</v>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="n">
+      <c r="A64" s="1" t="n">
         <v>43553</v>
       </c>
       <c r="B64" t="n">
         <v>0.01456866507753599</v>
       </c>
       <c r="C64" t="n">
-        <v>0.03494084912618518</v>
+        <v>0.03494084912618515</v>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="n">
+      <c r="A65" s="1" t="n">
         <v>43585</v>
       </c>
       <c r="B65" t="n">
         <v>0.03765434229152521</v>
       </c>
       <c r="C65" t="n">
-        <v>0.02737376576035038</v>
+        <v>0.0273737657603504</v>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="n">
+      <c r="A66" s="1" t="n">
         <v>43616</v>
       </c>
       <c r="B66" t="n">
         <v>-0.060324641374617</v>
       </c>
       <c r="C66" t="n">
-        <v>-0.02222157984850626</v>
+        <v>-0.02222157984850629</v>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="n">
+      <c r="A67" s="1" t="n">
         <v>43644</v>
       </c>
       <c r="B67" t="n">
         <v>0.07055400725002227</v>
       </c>
       <c r="C67" t="n">
-        <v>0.04186613772142071</v>
+        <v>0.04186613772142072</v>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="n">
+      <c r="A68" s="1" t="n">
         <v>43677</v>
       </c>
       <c r="B68" t="n">
         <v>0.00441979568404516</v>
       </c>
       <c r="C68" t="n">
-        <v>0.009522815551679515</v>
+        <v>0.009522815551679505</v>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="n">
+      <c r="A69" s="1" t="n">
         <v>43707</v>
       </c>
       <c r="B69" t="n">
         <v>-0.01853498241999796</v>
       </c>
       <c r="C69" t="n">
-        <v>0.01521033315853495</v>
+        <v>0.01521033315853493</v>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="n">
+      <c r="A70" s="1" t="n">
         <v>43738</v>
       </c>
       <c r="B70" t="n">
         <v>0.02461150917292742</v>
       </c>
       <c r="C70" t="n">
-        <v>0.006604812653261427</v>
+        <v>0.006604812653261434</v>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="n">
+      <c r="A71" s="1" t="n">
         <v>43769</v>
       </c>
       <c r="B71" t="n">
         <v>0.02195922871780593</v>
       </c>
       <c r="C71" t="n">
-        <v>-0.001327221783458395</v>
+        <v>-0.00132722178345838</v>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="n">
+      <c r="A72" s="1" t="n">
         <v>43798</v>
       </c>
       <c r="B72" t="n">
         <v>0.0298433572640832</v>
       </c>
       <c r="C72" t="n">
-        <v>0.01873125958053232</v>
+        <v>0.01873125958053234</v>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="n">
+      <c r="A73" s="1" t="n">
         <v>43830</v>
       </c>
       <c r="B73" t="n">
         <v>0.03494967527316942</v>
       </c>
       <c r="C73" t="n">
-        <v>0.04193944098221213</v>
+        <v>0.0419394409822121</v>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="n">
+      <c r="A74" s="1" t="n">
         <v>43861</v>
       </c>
       <c r="B74" t="n">
         <v>-0.009759123053471621</v>
       </c>
       <c r="C74" t="n">
-        <v>0.01169955204495741</v>
+        <v>0.0116995520449574</v>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="n">
+      <c r="A75" s="1" t="n">
         <v>43889</v>
       </c>
       <c r="B75" t="n">
         <v>-0.08796479084431257</v>
       </c>
       <c r="C75" t="n">
-        <v>-0.08547222154564432</v>
+        <v>-0.08547222154564435</v>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="n">
+      <c r="A76" s="1" t="n">
         <v>43921</v>
       </c>
       <c r="B76" t="n">
@@ -1277,7 +1263,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="n">
+      <c r="A77" s="1" t="n">
         <v>43951</v>
       </c>
       <c r="B77" t="n">
@@ -1288,18 +1274,18 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="n">
+      <c r="A78" s="1" t="n">
         <v>43980</v>
       </c>
       <c r="B78" t="n">
         <v>0.04154101329515191</v>
       </c>
       <c r="C78" t="n">
-        <v>0.02615620793453863</v>
+        <v>0.02615620793453864</v>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="n">
+      <c r="A79" s="1" t="n">
         <v>44012</v>
       </c>
       <c r="B79" t="n">
@@ -1310,40 +1296,40 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="n">
+      <c r="A80" s="1" t="n">
         <v>44043</v>
       </c>
       <c r="B80" t="n">
         <v>0.04862865623248207</v>
       </c>
       <c r="C80" t="n">
-        <v>0.07148084680712648</v>
+        <v>0.07148084680712646</v>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="2" t="n">
+      <c r="A81" s="1" t="n">
         <v>44074</v>
       </c>
       <c r="B81" t="n">
         <v>0.06545675104886525</v>
       </c>
       <c r="C81" t="n">
-        <v>0.03204056865028185</v>
+        <v>0.03204056865028183</v>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="n">
+      <c r="A82" s="1" t="n">
         <v>44104</v>
       </c>
       <c r="B82" t="n">
         <v>-0.03798501478694814</v>
       </c>
       <c r="C82" t="n">
-        <v>-0.0179282562867679</v>
+        <v>-0.01792825628676788</v>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="2" t="n">
+      <c r="A83" s="1" t="n">
         <v>44134</v>
       </c>
       <c r="B83" t="n">
@@ -1354,260 +1340,260 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="n">
+      <c r="A84" s="1" t="n">
         <v>44165</v>
       </c>
       <c r="B84" t="n">
         <v>0.1287856698772999</v>
       </c>
       <c r="C84" t="n">
-        <v>0.07259584873826552</v>
+        <v>0.07259584873826551</v>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="n">
+      <c r="A85" s="1" t="n">
         <v>44196</v>
       </c>
       <c r="B85" t="n">
         <v>0.03968201739931271</v>
       </c>
       <c r="C85" t="n">
-        <v>0.0289022890468589</v>
+        <v>0.02890228904685891</v>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="n">
+      <c r="A86" s="1" t="n">
         <v>44225</v>
       </c>
       <c r="B86" t="n">
         <v>-0.01188408970784299</v>
       </c>
       <c r="C86" t="n">
-        <v>-0.005280756260837319</v>
+        <v>-0.005280756260837304</v>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="2" t="n">
+      <c r="A87" s="1" t="n">
         <v>44253</v>
       </c>
       <c r="B87" t="n">
         <v>0.02723423490668533</v>
       </c>
       <c r="C87" t="n">
-        <v>-0.004671551493394119</v>
+        <v>-0.004671551493394105</v>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="2" t="n">
+      <c r="A88" s="1" t="n">
         <v>44286</v>
       </c>
       <c r="B88" t="n">
         <v>0.04553181616120811</v>
       </c>
       <c r="C88" t="n">
-        <v>0.08268309892796805</v>
+        <v>0.08268309892796803</v>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="2" t="n">
+      <c r="A89" s="1" t="n">
         <v>44316</v>
       </c>
       <c r="B89" t="n">
         <v>0.05011621462319103</v>
       </c>
       <c r="C89" t="n">
-        <v>0.02435557113386075</v>
+        <v>0.02435557113386077</v>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="n">
+      <c r="A90" s="1" t="n">
         <v>44347</v>
       </c>
       <c r="B90" t="n">
         <v>0.0203274953817251</v>
       </c>
       <c r="C90" t="n">
-        <v>0.02389959304873387</v>
+        <v>0.02389959304873388</v>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="2" t="n">
+      <c r="A91" s="1" t="n">
         <v>44377</v>
       </c>
       <c r="B91" t="n">
         <v>0.008869956342518076</v>
       </c>
       <c r="C91" t="n">
-        <v>-0.01678166711100587</v>
+        <v>-0.01678166711100586</v>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="2" t="n">
+      <c r="A92" s="1" t="n">
         <v>44407</v>
       </c>
       <c r="B92" t="n">
         <v>0.01871606001939291</v>
       </c>
       <c r="C92" t="n">
-        <v>0.02847485560076044</v>
+        <v>0.02847485560076045</v>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="2" t="n">
+      <c r="A93" s="1" t="n">
         <v>44439</v>
       </c>
       <c r="B93" t="n">
         <v>0.0227885548654776</v>
       </c>
       <c r="C93" t="n">
-        <v>0.007997307359006554</v>
+        <v>0.007997307359006561</v>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="2" t="n">
+      <c r="A94" s="1" t="n">
         <v>44469</v>
       </c>
       <c r="B94" t="n">
         <v>-0.04479491538928013</v>
       </c>
       <c r="C94" t="n">
-        <v>-0.05851167314004319</v>
+        <v>-0.05851167314004321</v>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="2" t="n">
+      <c r="A95" s="1" t="n">
         <v>44498</v>
       </c>
       <c r="B95" t="n">
         <v>0.06356405559391054</v>
       </c>
       <c r="C95" t="n">
-        <v>0.03511007569842588</v>
+        <v>0.0351100756984259</v>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="2" t="n">
+      <c r="A96" s="1" t="n">
         <v>44530</v>
       </c>
       <c r="B96" t="n">
         <v>-0.01499364534082952</v>
       </c>
       <c r="C96" t="n">
-        <v>-0.03091937213376149</v>
+        <v>-0.03091937213376151</v>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="2" t="n">
+      <c r="A97" s="1" t="n">
         <v>44561</v>
       </c>
       <c r="B97" t="n">
         <v>0.05277926573817891</v>
       </c>
       <c r="C97" t="n">
-        <v>0.08029407380856302</v>
+        <v>0.08029407380856303</v>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="2" t="n">
+      <c r="A98" s="1" t="n">
         <v>44592</v>
       </c>
       <c r="B98" t="n">
         <v>-0.04109160394901694</v>
       </c>
       <c r="C98" t="n">
-        <v>-0.01771171394965616</v>
+        <v>-0.01771171394965615</v>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="2" t="n">
+      <c r="A99" s="1" t="n">
         <v>44620</v>
       </c>
       <c r="B99" t="n">
         <v>-0.02413422789249773</v>
       </c>
       <c r="C99" t="n">
-        <v>-0.01250250203656948</v>
+        <v>-0.01250250203656946</v>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="2" t="n">
+      <c r="A100" s="1" t="n">
         <v>44651</v>
       </c>
       <c r="B100" t="n">
         <v>0.02747207877569881</v>
       </c>
       <c r="C100" t="n">
-        <v>0.04890168968953409</v>
+        <v>0.04890168968953411</v>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="2" t="n">
+      <c r="A101" s="1" t="n">
         <v>44680</v>
       </c>
       <c r="B101" t="n">
         <v>-0.07249985109846308</v>
       </c>
       <c r="C101" t="n">
-        <v>-0.03170811600039795</v>
+        <v>-0.03170811600039797</v>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="2" t="n">
+      <c r="A102" s="1" t="n">
         <v>44712</v>
       </c>
       <c r="B102" t="n">
         <v>0.005813538699808843</v>
       </c>
       <c r="C102" t="n">
-        <v>0.01033927945608507</v>
+        <v>0.01033927945608506</v>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="2" t="n">
+      <c r="A103" s="1" t="n">
         <v>44742</v>
       </c>
       <c r="B103" t="n">
         <v>-0.08621156652422018</v>
       </c>
       <c r="C103" t="n">
-        <v>-0.05498017284054231</v>
+        <v>-0.05498017284054228</v>
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="2" t="n">
+      <c r="A104" s="1" t="n">
         <v>44771</v>
       </c>
       <c r="B104" t="n">
         <v>0.07917156963943639</v>
       </c>
       <c r="C104" t="n">
-        <v>0.03594266589739632</v>
+        <v>0.03594266589739633</v>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="2" t="n">
+      <c r="A105" s="1" t="n">
         <v>44804</v>
       </c>
       <c r="B105" t="n">
         <v>-0.04330370505050581</v>
       </c>
       <c r="C105" t="n">
-        <v>-0.02659920566565774</v>
+        <v>-0.02659920566565771</v>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="2" t="n">
+      <c r="A106" s="1" t="n">
         <v>44834</v>
       </c>
       <c r="B106" t="n">
         <v>-0.0918304814629351</v>
       </c>
       <c r="C106" t="n">
-        <v>-0.08280019414302596</v>
+        <v>-0.08280019414302595</v>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="2" t="n">
+      <c r="A107" s="1" t="n">
         <v>44865</v>
       </c>
       <c r="B107" t="n">
@@ -1618,73 +1604,73 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="2" t="n">
+      <c r="A108" s="1" t="n">
         <v>44895</v>
       </c>
       <c r="B108" t="n">
         <v>0.07026136859463911</v>
       </c>
       <c r="C108" t="n">
-        <v>0.06016281139504846</v>
+        <v>0.06016281139504845</v>
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="2" t="n">
+      <c r="A109" s="1" t="n">
         <v>44925</v>
       </c>
       <c r="B109" t="n">
         <v>-0.04202625539539358</v>
       </c>
       <c r="C109" t="n">
-        <v>-0.02835811569867659</v>
+        <v>-0.02835811569867658</v>
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="2" t="n">
+      <c r="A110" s="1" t="n">
         <v>44957</v>
       </c>
       <c r="B110" t="n">
         <v>0.06632416178953368</v>
       </c>
       <c r="C110" t="n">
-        <v>0.02393514447393393</v>
+        <v>0.02393514447393395</v>
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="2" t="n">
+      <c r="A111" s="1" t="n">
         <v>44985</v>
       </c>
       <c r="B111" t="n">
         <v>-0.02251621511761719</v>
       </c>
       <c r="C111" t="n">
-        <v>-0.00689128081288972</v>
+        <v>-0.006891280812889715</v>
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="2" t="n">
+      <c r="A112" s="1" t="n">
         <v>45016</v>
       </c>
       <c r="B112" t="n">
         <v>0.03103550892661608</v>
       </c>
       <c r="C112" t="n">
-        <v>0.01184214150570381</v>
+        <v>0.01184214150570382</v>
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="2" t="n">
+      <c r="A113" s="1" t="n">
         <v>45044</v>
       </c>
       <c r="B113" t="n">
         <v>0.02629695395519377</v>
       </c>
       <c r="C113" t="n">
-        <v>0.02734082497437937</v>
+        <v>0.0273408249743794</v>
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="2" t="n">
+      <c r="A114" s="1" t="n">
         <v>45077</v>
       </c>
       <c r="B114" t="n">
@@ -1695,40 +1681,40 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="2" t="n">
+      <c r="A115" s="1" t="n">
         <v>45107</v>
       </c>
       <c r="B115" t="n">
         <v>0.06099850414882597</v>
       </c>
       <c r="C115" t="n">
-        <v>0.01631181051322895</v>
+        <v>0.01631181051322896</v>
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="2" t="n">
+      <c r="A116" s="1" t="n">
         <v>45138</v>
       </c>
       <c r="B116" t="n">
         <v>0.02926957614374468</v>
       </c>
       <c r="C116" t="n">
-        <v>0.008283814823725675</v>
+        <v>0.008283814823725677</v>
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="2" t="n">
+      <c r="A117" s="1" t="n">
         <v>45169</v>
       </c>
       <c r="B117" t="n">
         <v>-0.02254274830541499</v>
       </c>
       <c r="C117" t="n">
-        <v>-0.02450943501530417</v>
+        <v>-0.02450943501530415</v>
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="2" t="n">
+      <c r="A118" s="1" t="n">
         <v>45198</v>
       </c>
       <c r="B118" t="n">
@@ -1739,139 +1725,139 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="2" t="n">
+      <c r="A119" s="1" t="n">
         <v>45230</v>
       </c>
       <c r="B119" t="n">
         <v>-0.0218263884926712</v>
       </c>
       <c r="C119" t="n">
-        <v>-0.01101723542670296</v>
+        <v>-0.01101723542670293</v>
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="2" t="n">
+      <c r="A120" s="1" t="n">
         <v>45260</v>
       </c>
       <c r="B120" t="n">
         <v>0.09032959900387923</v>
       </c>
       <c r="C120" t="n">
-        <v>0.03459969159971099</v>
+        <v>0.034599691599711</v>
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="2" t="n">
+      <c r="A121" s="1" t="n">
         <v>45289</v>
       </c>
       <c r="B121" t="n">
         <v>0.04518290595522654</v>
       </c>
       <c r="C121" t="n">
-        <v>0.0190837411773818</v>
+        <v>0.01908374117738178</v>
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="2" t="n">
+      <c r="A122" s="1" t="n">
         <v>45322</v>
       </c>
       <c r="B122" t="n">
         <v>0.01223860433047028</v>
       </c>
       <c r="C122" t="n">
-        <v>-0.002972561984548157</v>
+        <v>-0.002972561984548129</v>
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="2" t="n">
+      <c r="A123" s="1" t="n">
         <v>45351</v>
       </c>
       <c r="B123" t="n">
         <v>0.039045010282345</v>
       </c>
       <c r="C123" t="n">
-        <v>0.02182263764553106</v>
+        <v>0.02182263764553105</v>
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="2" t="n">
+      <c r="A124" s="1" t="n">
         <v>45380</v>
       </c>
       <c r="B124" t="n">
         <v>0.0364210345677266</v>
       </c>
       <c r="C124" t="n">
-        <v>0.02766588670083584</v>
+        <v>0.02766588670083583</v>
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="2" t="n">
+      <c r="A125" s="1" t="n">
         <v>45412</v>
       </c>
       <c r="B125" t="n">
         <v>-0.03611535468175369</v>
       </c>
       <c r="C125" t="n">
-        <v>0.007887485409802903</v>
+        <v>0.007887485409802896</v>
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="2" t="n">
+      <c r="A126" s="1" t="n">
         <v>45443</v>
       </c>
       <c r="B126" t="n">
         <v>0.05170302879334956</v>
       </c>
       <c r="C126" t="n">
-        <v>0.03008781794761483</v>
+        <v>0.03008781794761482</v>
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="2" t="n">
+      <c r="A127" s="1" t="n">
         <v>45471</v>
       </c>
       <c r="B127" t="n">
         <v>0.01658165662881855</v>
       </c>
       <c r="C127" t="n">
-        <v>-0.01003117137510178</v>
+        <v>-0.01003117137510176</v>
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="2" t="n">
+      <c r="A128" s="1" t="n">
         <v>45504</v>
       </c>
       <c r="B128" t="n">
         <v>0.01644259091919383</v>
       </c>
       <c r="C128" t="n">
-        <v>0.02739986639078621</v>
+        <v>0.0273998663907862</v>
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="2" t="n">
+      <c r="A129" s="1" t="n">
         <v>45534</v>
       </c>
       <c r="B129" t="n">
         <v>0.02656573967480293</v>
       </c>
       <c r="C129" t="n">
-        <v>0.04480272094453805</v>
+        <v>0.04480272094453803</v>
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="2" t="n">
+      <c r="A130" s="1" t="n">
         <v>45565</v>
       </c>
       <c r="B130" t="n">
         <v>0.01494857097512915</v>
       </c>
       <c r="C130" t="n">
-        <v>-0.005980811556354734</v>
+        <v>-0.005980811556354736</v>
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="2" t="n">
+      <c r="A131" s="1" t="n">
         <v>45596</v>
       </c>
       <c r="B131" t="n">
@@ -1882,18 +1868,18 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="2" t="n">
+      <c r="A132" s="1" t="n">
         <v>45625</v>
       </c>
       <c r="B132" t="n">
         <v>0.04148309969298379</v>
       </c>
       <c r="C132" t="n">
-        <v>-6.588281982651024e-05</v>
+        <v>-6.588281982651198e-05</v>
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="2" t="n">
+      <c r="A133" s="1" t="n">
         <v>45657</v>
       </c>
       <c r="B133" t="n">
@@ -1904,106 +1890,106 @@
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="2" t="n">
+      <c r="A134" s="1" t="n">
         <v>45688</v>
       </c>
       <c r="B134" t="n">
         <v>0.0307856990220507</v>
       </c>
       <c r="C134" t="n">
-        <v>-0.001859581680386343</v>
+        <v>-0.001859581680386347</v>
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="2" t="n">
+      <c r="A135" s="1" t="n">
         <v>45716</v>
       </c>
       <c r="B135" t="n">
         <v>0.005323365436410136</v>
       </c>
       <c r="C135" t="n">
-        <v>0.009739061651612407</v>
+        <v>0.009739061651612401</v>
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="2" t="n">
+      <c r="A136" s="1" t="n">
         <v>45747</v>
       </c>
       <c r="B136" t="n">
         <v>-0.03930165295658457</v>
       </c>
       <c r="C136" t="n">
-        <v>0.01506767380717352</v>
+        <v>0.01506767380717351</v>
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="2" t="n">
+      <c r="A137" s="1" t="n">
         <v>45777</v>
       </c>
       <c r="B137" t="n">
         <v>-0.0004032469247518319</v>
       </c>
       <c r="C137" t="n">
-        <v>0.0399268407866919</v>
+        <v>0.03992684078669188</v>
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="2" t="n">
+      <c r="A138" s="1" t="n">
         <v>45807</v>
       </c>
       <c r="B138" t="n">
         <v>0.0504861113117907</v>
       </c>
       <c r="C138" t="n">
-        <v>-0.01199337100743361</v>
+        <v>-0.0119933710074336</v>
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="2" t="n">
+      <c r="A139" s="1" t="n">
         <v>45838</v>
       </c>
       <c r="B139" t="n">
         <v>0.04362568245725708</v>
       </c>
       <c r="C139" t="n">
-        <v>0.001485880928199708</v>
+        <v>0.001485880928199699</v>
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="2" t="n">
+      <c r="A140" s="1" t="n">
         <v>45869</v>
       </c>
       <c r="B140" t="n">
         <v>0.01701146208277682</v>
       </c>
       <c r="C140" t="n">
-        <v>-0.005234222240507071</v>
+        <v>-0.005234222240507087</v>
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="2" t="n">
+      <c r="A141" s="1" t="n">
         <v>45898</v>
       </c>
       <c r="B141" t="n">
         <v>0.02374663315104465</v>
       </c>
       <c r="C141" t="n">
-        <v>0.01386896406975188</v>
+        <v>0.0138689640697519</v>
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="2" t="n">
+      <c r="A142" s="1" t="n">
         <v>45930</v>
       </c>
       <c r="B142" t="n">
         <v>0.02754083678244896</v>
       </c>
       <c r="C142" t="n">
-        <v>0.0006082066964267895</v>
+        <v>0.0006082066964267748</v>
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="2" t="n">
+      <c r="A143" s="1" t="n">
         <v>45961</v>
       </c>
       <c r="B143" t="n">
@@ -2014,25 +2000,25 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="2" t="n">
+      <c r="A144" s="1" t="n">
         <v>45989</v>
       </c>
       <c r="B144" t="n">
         <v>0.00741020528526478</v>
       </c>
       <c r="C144" t="n">
-        <v>0.05065362269007078</v>
+        <v>0.05065362269007079</v>
       </c>
     </row>
     <row r="145">
-      <c r="A145" s="2" t="n">
+      <c r="A145" s="1" t="n">
         <v>46022</v>
       </c>
       <c r="B145" t="n">
         <v>0.01455154193474042</v>
       </c>
       <c r="C145" t="n">
-        <v>0.008039240061955099</v>
+        <v>0.008039240061955111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>